<commit_message>
✅ Veri Güncellendi:  - Tue Mar  3 01:26:51 UTC 2026
</commit_message>
<xml_diff>
--- a/leads_output.xlsx
+++ b/leads_output.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E269"/>
+  <dimension ref="A1:E281"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -8220,6 +8220,354 @@
         </is>
       </c>
     </row>
+    <row r="270">
+      <c r="A270" t="inlineStr">
+        <is>
+          <t>AYLİN ECZANESİ</t>
+        </is>
+      </c>
+      <c r="B270" t="inlineStr">
+        <is>
+          <t>
++90 216 545 03 23</t>
+        </is>
+      </c>
+      <c r="C270" t="inlineStr">
+        <is>
+          <t>
+Koşuyolu, Koşuyolu Cd. NO:95/A, 34718 Kadıköy/İstanbul, Türkiye</t>
+        </is>
+      </c>
+      <c r="D270" t="inlineStr">
+        <is>
+          <t>Kadikoy/Istanbul</t>
+        </is>
+      </c>
+      <c r="E270" t="inlineStr">
+        <is>
+          <t>2026-03-03 01:26</t>
+        </is>
+      </c>
+    </row>
+    <row r="271">
+      <c r="A271" t="inlineStr">
+        <is>
+          <t>Elif Eczanesi</t>
+        </is>
+      </c>
+      <c r="B271" t="inlineStr">
+        <is>
+          <t>
++90 216 478 09 90</t>
+        </is>
+      </c>
+      <c r="C271" t="inlineStr">
+        <is>
+          <t>
+Rize Girişenler Sitesİ, 19 Mayıs Mh, Mehpare Sokağı 18/1, 34736 Kadıköy/İstanbul, Türkiye</t>
+        </is>
+      </c>
+      <c r="D271" t="inlineStr">
+        <is>
+          <t>Kadikoy/Istanbul</t>
+        </is>
+      </c>
+      <c r="E271" t="inlineStr">
+        <is>
+          <t>2026-03-03 01:26</t>
+        </is>
+      </c>
+    </row>
+    <row r="272">
+      <c r="A272" t="inlineStr">
+        <is>
+          <t>Elit Plus Eczanesi</t>
+        </is>
+      </c>
+      <c r="B272" t="inlineStr">
+        <is>
+          <t>
++90 216 411 20 20</t>
+        </is>
+      </c>
+      <c r="C272" t="inlineStr">
+        <is>
+          <t>
+Caddebostan, Bağdat Cad. no:306/A, 34728 Kadıköy/İstanbul, Türkiye</t>
+        </is>
+      </c>
+      <c r="D272" t="inlineStr">
+        <is>
+          <t>Kadikoy/Istanbul</t>
+        </is>
+      </c>
+      <c r="E272" t="inlineStr">
+        <is>
+          <t>2026-03-03 01:26</t>
+        </is>
+      </c>
+    </row>
+    <row r="273">
+      <c r="A273" t="inlineStr">
+        <is>
+          <t>Erengül Eczanesi</t>
+        </is>
+      </c>
+      <c r="B273" t="inlineStr">
+        <is>
+          <t>
++90 216 418 69 36</t>
+        </is>
+      </c>
+      <c r="C273" t="inlineStr">
+        <is>
+          <t>
+Osmanağa, Hasırcı Başı Cd 3/A, 34714 Kadıköy/İstanbul, Türkiye</t>
+        </is>
+      </c>
+      <c r="D273" t="inlineStr">
+        <is>
+          <t>Kadikoy/Istanbul</t>
+        </is>
+      </c>
+      <c r="E273" t="inlineStr">
+        <is>
+          <t>2026-03-03 01:26</t>
+        </is>
+      </c>
+    </row>
+    <row r="274">
+      <c r="A274" t="inlineStr">
+        <is>
+          <t>Beyaz Köşk Eczanesi Kızıltoprak</t>
+        </is>
+      </c>
+      <c r="B274" t="inlineStr">
+        <is>
+          <t>
++90 552 697 30 20</t>
+        </is>
+      </c>
+      <c r="C274" t="inlineStr">
+        <is>
+          <t>
+Feneryolu, Bağdat Cad. No:61/A, 34724 Kadıköy/İstanbul, Türkiye</t>
+        </is>
+      </c>
+      <c r="D274" t="inlineStr">
+        <is>
+          <t>Kadikoy/Istanbul</t>
+        </is>
+      </c>
+      <c r="E274" t="inlineStr">
+        <is>
+          <t>2026-03-03 01:26</t>
+        </is>
+      </c>
+    </row>
+    <row r="275">
+      <c r="A275" t="inlineStr">
+        <is>
+          <t>Yenişehir Eczanesi</t>
+        </is>
+      </c>
+      <c r="B275" t="inlineStr">
+        <is>
+          <t>
++90 216 302 72 70</t>
+        </is>
+      </c>
+      <c r="C275" t="inlineStr">
+        <is>
+          <t>
+Göztepe, Tütüncü Mehmet Efendi Cd. No:10/C, 34730 Kadıköy/İstanbul, Türkiye</t>
+        </is>
+      </c>
+      <c r="D275" t="inlineStr">
+        <is>
+          <t>Kadikoy/Istanbul</t>
+        </is>
+      </c>
+      <c r="E275" t="inlineStr">
+        <is>
+          <t>2026-03-03 01:26</t>
+        </is>
+      </c>
+    </row>
+    <row r="276">
+      <c r="A276" t="inlineStr">
+        <is>
+          <t>FİTO ECZANESİ</t>
+        </is>
+      </c>
+      <c r="B276" t="inlineStr">
+        <is>
+          <t>
++90 216 418 44 15</t>
+        </is>
+      </c>
+      <c r="C276" t="inlineStr">
+        <is>
+          <t>
+Hasanpaşa, Söğütlüçeşme Cad. söğütlü han D:178/A, 34722 Kadıköy/İstanbul, Türkiye</t>
+        </is>
+      </c>
+      <c r="D276" t="inlineStr">
+        <is>
+          <t>Kadikoy/Istanbul</t>
+        </is>
+      </c>
+      <c r="E276" t="inlineStr">
+        <is>
+          <t>2026-03-03 01:26</t>
+        </is>
+      </c>
+    </row>
+    <row r="277">
+      <c r="A277" t="inlineStr">
+        <is>
+          <t>Renk Eczanesi</t>
+        </is>
+      </c>
+      <c r="B277" t="inlineStr">
+        <is>
+          <t>
++90 216 755 40 50</t>
+        </is>
+      </c>
+      <c r="C277" t="inlineStr">
+        <is>
+          <t>
+Göztepe, Karanfil Sk. 24A D:B, 34730 Kadıköy/İstanbul, Türkiye</t>
+        </is>
+      </c>
+      <c r="D277" t="inlineStr">
+        <is>
+          <t>Kadikoy/Istanbul</t>
+        </is>
+      </c>
+      <c r="E277" t="inlineStr">
+        <is>
+          <t>2026-03-03 01:26</t>
+        </is>
+      </c>
+    </row>
+    <row r="278">
+      <c r="A278" t="inlineStr">
+        <is>
+          <t>Anık Eczanesi</t>
+        </is>
+      </c>
+      <c r="B278" t="inlineStr">
+        <is>
+          <t>
++90 216 408 12 50</t>
+        </is>
+      </c>
+      <c r="C278" t="inlineStr">
+        <is>
+          <t>
+19 Mayıs Mahallesi Bayar Caddesi, 14/1 Ondokuzmayıs/Kadıköy/İstanbul, 34736, Türkiye</t>
+        </is>
+      </c>
+      <c r="D278" t="inlineStr">
+        <is>
+          <t>Kadikoy/Istanbul</t>
+        </is>
+      </c>
+      <c r="E278" t="inlineStr">
+        <is>
+          <t>2026-03-03 01:26</t>
+        </is>
+      </c>
+    </row>
+    <row r="279">
+      <c r="A279" t="inlineStr">
+        <is>
+          <t>Eczane İpek</t>
+        </is>
+      </c>
+      <c r="B279" t="inlineStr">
+        <is>
+          <t>
++90 216 347 96 46</t>
+        </is>
+      </c>
+      <c r="C279" t="inlineStr">
+        <is>
+          <t>
+Zühtüpaşa, Hasan Amir Sk. Bayrak Apt. D:11/A, 34724 Kadıköy/İstanbul, Türkiye</t>
+        </is>
+      </c>
+      <c r="D279" t="inlineStr">
+        <is>
+          <t>Kadikoy/Istanbul</t>
+        </is>
+      </c>
+      <c r="E279" t="inlineStr">
+        <is>
+          <t>2026-03-03 01:26</t>
+        </is>
+      </c>
+    </row>
+    <row r="280">
+      <c r="A280" t="inlineStr">
+        <is>
+          <t>SuadiyeSu Eczanesi</t>
+        </is>
+      </c>
+      <c r="B280" t="inlineStr">
+        <is>
+          <t>
++90 216 373 46 33</t>
+        </is>
+      </c>
+      <c r="C280" t="inlineStr">
+        <is>
+          <t>
+Suadiye, Bağdat Cad. No:428/B, 34740 Kadıköy/İstanbul, Türkiye</t>
+        </is>
+      </c>
+      <c r="D280" t="inlineStr">
+        <is>
+          <t>Kadikoy/Istanbul</t>
+        </is>
+      </c>
+      <c r="E280" t="inlineStr">
+        <is>
+          <t>2026-03-03 01:26</t>
+        </is>
+      </c>
+    </row>
+    <row r="281">
+      <c r="A281" t="inlineStr">
+        <is>
+          <t>Tülay Eczanesi</t>
+        </is>
+      </c>
+      <c r="B281" t="inlineStr">
+        <is>
+          <t>
++90 216 337 52 65</t>
+        </is>
+      </c>
+      <c r="C281" t="inlineStr">
+        <is>
+          <t>
+Eğitim, Nahitbey Sok. No:62, 34722 Kadıköy/İstanbul, Türkiye</t>
+        </is>
+      </c>
+      <c r="D281" t="inlineStr">
+        <is>
+          <t>Kadikoy/Istanbul</t>
+        </is>
+      </c>
+      <c r="E281" t="inlineStr">
+        <is>
+          <t>2026-03-03 01:26</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
✅ Veri Güncellendi:  - Wed Mar  4 01:21:22 UTC 2026
</commit_message>
<xml_diff>
--- a/leads_output.xlsx
+++ b/leads_output.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E281"/>
+  <dimension ref="A1:E283"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -8568,6 +8568,64 @@
         </is>
       </c>
     </row>
+    <row r="282">
+      <c r="A282" t="inlineStr">
+        <is>
+          <t>Yeldeğirmeni Eczanesi Aktif</t>
+        </is>
+      </c>
+      <c r="B282" t="inlineStr">
+        <is>
+          <t>
++90 544 378 23 80</t>
+        </is>
+      </c>
+      <c r="C282" t="inlineStr">
+        <is>
+          <t>
+Rasimpaşa, Karakolhane Cd. No 9A, 34716 Kadıköy/İstanbul, Türkiye</t>
+        </is>
+      </c>
+      <c r="D282" t="inlineStr">
+        <is>
+          <t>Kadikoy/Istanbul</t>
+        </is>
+      </c>
+      <c r="E282" t="inlineStr">
+        <is>
+          <t>2026-03-04 01:21</t>
+        </is>
+      </c>
+    </row>
+    <row r="283">
+      <c r="A283" t="inlineStr">
+        <is>
+          <t>Fortis Eczanesi</t>
+        </is>
+      </c>
+      <c r="B283" t="inlineStr">
+        <is>
+          <t>
++90 531 886 89 00</t>
+        </is>
+      </c>
+      <c r="C283" t="inlineStr">
+        <is>
+          <t>
+Fikirtepe, Yıldırım Sk. No:2, 34720 Kadıköy/İstanbul, Türkiye</t>
+        </is>
+      </c>
+      <c r="D283" t="inlineStr">
+        <is>
+          <t>Kadikoy/Istanbul</t>
+        </is>
+      </c>
+      <c r="E283" t="inlineStr">
+        <is>
+          <t>2026-03-04 01:21</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
✅ Veri Güncellendi:  - Thu Mar  5 01:24:55 UTC 2026
</commit_message>
<xml_diff>
--- a/leads_output.xlsx
+++ b/leads_output.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E283"/>
+  <dimension ref="A1:E300"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -8626,6 +8626,498 @@
         </is>
       </c>
     </row>
+    <row r="284">
+      <c r="A284" t="inlineStr">
+        <is>
+          <t>Eczane Miray Yılmaz</t>
+        </is>
+      </c>
+      <c r="B284" t="inlineStr">
+        <is>
+          <t>
++90 216 350 49 50</t>
+        </is>
+      </c>
+      <c r="C284" t="inlineStr">
+        <is>
+          <t>
+Erenköy, Ethemefendi Caddesi No:59 D:F, 34738 Kadıköy/İstanbul, Türkiye</t>
+        </is>
+      </c>
+      <c r="D284" t="inlineStr">
+        <is>
+          <t>Kadikoy/Istanbul</t>
+        </is>
+      </c>
+      <c r="E284" t="inlineStr">
+        <is>
+          <t>2026-03-05 01:23</t>
+        </is>
+      </c>
+    </row>
+    <row r="285">
+      <c r="A285" t="inlineStr">
+        <is>
+          <t>Saraçoğlu Eczanesi</t>
+        </is>
+      </c>
+      <c r="B285" t="inlineStr">
+        <is>
+          <t>
++90 216 348 19 97</t>
+        </is>
+      </c>
+      <c r="C285" t="inlineStr">
+        <is>
+          <t>
+Eğitim, Fahrettin Kerim Gökay Cd no:115a, 34010 Kadıköy/İstanbul, Türkiye</t>
+        </is>
+      </c>
+      <c r="D285" t="inlineStr">
+        <is>
+          <t>Kadikoy/Istanbul</t>
+        </is>
+      </c>
+      <c r="E285" t="inlineStr">
+        <is>
+          <t>2026-03-05 01:23</t>
+        </is>
+      </c>
+    </row>
+    <row r="286">
+      <c r="A286" t="inlineStr">
+        <is>
+          <t>Eczane Turkuaz</t>
+        </is>
+      </c>
+      <c r="B286" t="inlineStr">
+        <is>
+          <t>
++90 216 566 06 78</t>
+        </is>
+      </c>
+      <c r="C286" t="inlineStr">
+        <is>
+          <t>
+Merdivenköy, Ressam Salih Erimez Cad No:7 D:5, 34732 Kadıköy/İstanbul, Türkiye</t>
+        </is>
+      </c>
+      <c r="D286" t="inlineStr">
+        <is>
+          <t>Kadikoy/Istanbul</t>
+        </is>
+      </c>
+      <c r="E286" t="inlineStr">
+        <is>
+          <t>2026-03-05 01:23</t>
+        </is>
+      </c>
+    </row>
+    <row r="287">
+      <c r="A287" t="inlineStr">
+        <is>
+          <t>ECZANE AKADEMİ</t>
+        </is>
+      </c>
+      <c r="B287" t="inlineStr">
+        <is>
+          <t>
++90 216 336 54 61</t>
+        </is>
+      </c>
+      <c r="C287" t="inlineStr">
+        <is>
+          <t>
+Rasimpaşa, Haydarpaşa Garı Yolu 4/A, 34716 Kadıköy/İstanbul, Türkiye</t>
+        </is>
+      </c>
+      <c r="D287" t="inlineStr">
+        <is>
+          <t>Kadikoy/Istanbul</t>
+        </is>
+      </c>
+      <c r="E287" t="inlineStr">
+        <is>
+          <t>2026-03-05 01:23</t>
+        </is>
+      </c>
+    </row>
+    <row r="288">
+      <c r="A288" t="inlineStr">
+        <is>
+          <t>Esra Eczanesi</t>
+        </is>
+      </c>
+      <c r="B288" t="inlineStr">
+        <is>
+          <t>
++90 216 340 33 44</t>
+        </is>
+      </c>
+      <c r="C288" t="inlineStr">
+        <is>
+          <t>
+Hasanpaşa, 34722 Kadıköy/İstanbul, Türkiye</t>
+        </is>
+      </c>
+      <c r="D288" t="inlineStr">
+        <is>
+          <t>Kadikoy/Istanbul</t>
+        </is>
+      </c>
+      <c r="E288" t="inlineStr">
+        <is>
+          <t>2026-03-05 01:23</t>
+        </is>
+      </c>
+    </row>
+    <row r="289">
+      <c r="A289" t="inlineStr">
+        <is>
+          <t>İDİL ECZANESİ</t>
+        </is>
+      </c>
+      <c r="B289" t="inlineStr">
+        <is>
+          <t>
++90 216 566 46 17</t>
+        </is>
+      </c>
+      <c r="C289" t="inlineStr">
+        <is>
+          <t>Yok</t>
+        </is>
+      </c>
+      <c r="D289" t="inlineStr">
+        <is>
+          <t>Kadikoy/Istanbul</t>
+        </is>
+      </c>
+      <c r="E289" t="inlineStr">
+        <is>
+          <t>2026-03-05 01:24</t>
+        </is>
+      </c>
+    </row>
+    <row r="290">
+      <c r="A290" t="inlineStr">
+        <is>
+          <t>Eczane Pamuk</t>
+        </is>
+      </c>
+      <c r="B290" t="inlineStr">
+        <is>
+          <t>
++90 216 565 09 74</t>
+        </is>
+      </c>
+      <c r="C290" t="inlineStr">
+        <is>
+          <t>
+Göztepe, Mustafa Mazhar Bey Sokağı No:24 D:B, 34730 Kadıköy/İstanbul, Türkiye</t>
+        </is>
+      </c>
+      <c r="D290" t="inlineStr">
+        <is>
+          <t>Kadikoy/Istanbul</t>
+        </is>
+      </c>
+      <c r="E290" t="inlineStr">
+        <is>
+          <t>2026-03-05 01:24</t>
+        </is>
+      </c>
+    </row>
+    <row r="291">
+      <c r="A291" t="inlineStr">
+        <is>
+          <t>Eczane Ozan</t>
+        </is>
+      </c>
+      <c r="B291" t="inlineStr">
+        <is>
+          <t>
++90 216 405 16 75</t>
+        </is>
+      </c>
+      <c r="C291" t="inlineStr">
+        <is>
+          <t>
+Caferağa, Ressam Şeref Akdik Sokağı No:3, 34714 Kadıköy/İstanbul, Türkiye</t>
+        </is>
+      </c>
+      <c r="D291" t="inlineStr">
+        <is>
+          <t>Kadikoy/Istanbul</t>
+        </is>
+      </c>
+      <c r="E291" t="inlineStr">
+        <is>
+          <t>2026-03-05 01:24</t>
+        </is>
+      </c>
+    </row>
+    <row r="292">
+      <c r="A292" t="inlineStr">
+        <is>
+          <t>anadolu eczanesi acıbadem</t>
+        </is>
+      </c>
+      <c r="B292" t="inlineStr">
+        <is>
+          <t>
++90 216 339 15 77</t>
+        </is>
+      </c>
+      <c r="C292" t="inlineStr">
+        <is>
+          <t>
+Acıbadem, Asalet Sk. 6/85, 34718 Kadıköy/İstanbul, Türkiye</t>
+        </is>
+      </c>
+      <c r="D292" t="inlineStr">
+        <is>
+          <t>Kadikoy/Istanbul</t>
+        </is>
+      </c>
+      <c r="E292" t="inlineStr">
+        <is>
+          <t>2026-03-05 01:24</t>
+        </is>
+      </c>
+    </row>
+    <row r="293">
+      <c r="A293" t="inlineStr">
+        <is>
+          <t>Eczane Mine</t>
+        </is>
+      </c>
+      <c r="B293" t="inlineStr">
+        <is>
+          <t>
++90 216 330 58 57</t>
+        </is>
+      </c>
+      <c r="C293" t="inlineStr">
+        <is>
+          <t>
+Caferağa, Moda Cd. No:92/B, 34710 Kadıköy/İstanbul, Türkiye</t>
+        </is>
+      </c>
+      <c r="D293" t="inlineStr">
+        <is>
+          <t>Kadikoy/Istanbul</t>
+        </is>
+      </c>
+      <c r="E293" t="inlineStr">
+        <is>
+          <t>2026-03-05 01:24</t>
+        </is>
+      </c>
+    </row>
+    <row r="294">
+      <c r="A294" t="inlineStr">
+        <is>
+          <t>Eczane Eylül</t>
+        </is>
+      </c>
+      <c r="B294" t="inlineStr">
+        <is>
+          <t>
++90 216 550 71 75</t>
+        </is>
+      </c>
+      <c r="C294" t="inlineStr">
+        <is>
+          <t>
+Hasanpaşa, Fahrettin Kerim Gökay Cd No:61 D:1, 34722 Kadıköy/İstanbul - Asya, Türkiye</t>
+        </is>
+      </c>
+      <c r="D294" t="inlineStr">
+        <is>
+          <t>Kadikoy/Istanbul</t>
+        </is>
+      </c>
+      <c r="E294" t="inlineStr">
+        <is>
+          <t>2026-03-05 01:24</t>
+        </is>
+      </c>
+    </row>
+    <row r="295">
+      <c r="A295" t="inlineStr">
+        <is>
+          <t>Eczane Serap</t>
+        </is>
+      </c>
+      <c r="B295" t="inlineStr">
+        <is>
+          <t>
++90 216 414 19 74</t>
+        </is>
+      </c>
+      <c r="C295" t="inlineStr">
+        <is>
+          <t>
+Eğitim, Kasrı Ali Cd. No:1, 34733 Kadıköy/İstanbul, Türkiye</t>
+        </is>
+      </c>
+      <c r="D295" t="inlineStr">
+        <is>
+          <t>Kadikoy/Istanbul</t>
+        </is>
+      </c>
+      <c r="E295" t="inlineStr">
+        <is>
+          <t>2026-03-05 01:24</t>
+        </is>
+      </c>
+    </row>
+    <row r="296">
+      <c r="A296" t="inlineStr">
+        <is>
+          <t>Mariposa Eczanesi</t>
+        </is>
+      </c>
+      <c r="B296" t="inlineStr">
+        <is>
+          <t>
++90 507 114 44 23</t>
+        </is>
+      </c>
+      <c r="C296" t="inlineStr">
+        <is>
+          <t>
+Albaraka bankası bitişiği, Rasimpaşa, Rıhtım Cd. No:46/A, 34716 Kadıköy/İstanbul, Türkiye</t>
+        </is>
+      </c>
+      <c r="D296" t="inlineStr">
+        <is>
+          <t>Kadikoy/Istanbul</t>
+        </is>
+      </c>
+      <c r="E296" t="inlineStr">
+        <is>
+          <t>2026-03-05 01:24</t>
+        </is>
+      </c>
+    </row>
+    <row r="297">
+      <c r="A297" t="inlineStr">
+        <is>
+          <t>Çağla Eczanesi</t>
+        </is>
+      </c>
+      <c r="B297" t="inlineStr">
+        <is>
+          <t>
++90 216 464 33 30</t>
+        </is>
+      </c>
+      <c r="C297" t="inlineStr">
+        <is>
+          <t>
+19 Mayıs Mahallesi Sinan Ercan Caddesi No:6 Kazasker, 34736 Kadıköy, Türkiye</t>
+        </is>
+      </c>
+      <c r="D297" t="inlineStr">
+        <is>
+          <t>Kadikoy/Istanbul</t>
+        </is>
+      </c>
+      <c r="E297" t="inlineStr">
+        <is>
+          <t>2026-03-05 01:24</t>
+        </is>
+      </c>
+    </row>
+    <row r="298">
+      <c r="A298" t="inlineStr">
+        <is>
+          <t>İlke Eczanesi</t>
+        </is>
+      </c>
+      <c r="B298" t="inlineStr">
+        <is>
+          <t>
++90 216 372 74 80</t>
+        </is>
+      </c>
+      <c r="C298" t="inlineStr">
+        <is>
+          <t>
+Balkan Apartmanı, Bostancı, Balkan Sk. 6/A, 34744 Kadıköy/İstanbul, Türkiye</t>
+        </is>
+      </c>
+      <c r="D298" t="inlineStr">
+        <is>
+          <t>Kadikoy/Istanbul</t>
+        </is>
+      </c>
+      <c r="E298" t="inlineStr">
+        <is>
+          <t>2026-03-05 01:24</t>
+        </is>
+      </c>
+    </row>
+    <row r="299">
+      <c r="A299" t="inlineStr">
+        <is>
+          <t>Vera Eczanesi</t>
+        </is>
+      </c>
+      <c r="B299" t="inlineStr">
+        <is>
+          <t>
++90 216 340 76 24</t>
+        </is>
+      </c>
+      <c r="C299" t="inlineStr">
+        <is>
+          <t>
+Acıbadem, Salah Birsel Sk., 34718 Kadıköy/İstanbul, Türkiye</t>
+        </is>
+      </c>
+      <c r="D299" t="inlineStr">
+        <is>
+          <t>Kadikoy/Istanbul</t>
+        </is>
+      </c>
+      <c r="E299" t="inlineStr">
+        <is>
+          <t>2026-03-05 01:24</t>
+        </is>
+      </c>
+    </row>
+    <row r="300">
+      <c r="A300" t="inlineStr">
+        <is>
+          <t>Eczane Fenerbahçe</t>
+        </is>
+      </c>
+      <c r="B300" t="inlineStr">
+        <is>
+          <t>
++90 216 336 96 51</t>
+        </is>
+      </c>
+      <c r="C300" t="inlineStr">
+        <is>
+          <t>
+Fenerbahçe, Operatör Cemil Topuzlu Cd. No:2 D:B, 34726 Kadıköy/İstanbul, Türkiye</t>
+        </is>
+      </c>
+      <c r="D300" t="inlineStr">
+        <is>
+          <t>Kadikoy/Istanbul</t>
+        </is>
+      </c>
+      <c r="E300" t="inlineStr">
+        <is>
+          <t>2026-03-05 01:24</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
✅ Veri Güncellendi:  - Fri Mar  6 01:26:17 UTC 2026
</commit_message>
<xml_diff>
--- a/leads_output.xlsx
+++ b/leads_output.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E300"/>
+  <dimension ref="A1:E302"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -9118,6 +9118,64 @@
         </is>
       </c>
     </row>
+    <row r="301">
+      <c r="A301" t="inlineStr">
+        <is>
+          <t>Fikirtepe Ihlamur Eczanesi</t>
+        </is>
+      </c>
+      <c r="B301" t="inlineStr">
+        <is>
+          <t>
++90 216 551 71 48</t>
+        </is>
+      </c>
+      <c r="C301" t="inlineStr">
+        <is>
+          <t>
+Fikirtepe, Volkan Sk. No:31-41/A, 34720 Kadıköy/İstanbul, Türkiye</t>
+        </is>
+      </c>
+      <c r="D301" t="inlineStr">
+        <is>
+          <t>Kadikoy/Istanbul</t>
+        </is>
+      </c>
+      <c r="E301" t="inlineStr">
+        <is>
+          <t>2026-03-06 01:26</t>
+        </is>
+      </c>
+    </row>
+    <row r="302">
+      <c r="A302" t="inlineStr">
+        <is>
+          <t>URAZ ECZANESİ</t>
+        </is>
+      </c>
+      <c r="B302" t="inlineStr">
+        <is>
+          <t>
++90 216 515 85 15</t>
+        </is>
+      </c>
+      <c r="C302" t="inlineStr">
+        <is>
+          <t>
+Erenköy, Ethemefendi Caddesi NO:108B, 34738 Kadıköy/İstanbul, Türkiye</t>
+        </is>
+      </c>
+      <c r="D302" t="inlineStr">
+        <is>
+          <t>Kadikoy/Istanbul</t>
+        </is>
+      </c>
+      <c r="E302" t="inlineStr">
+        <is>
+          <t>2026-03-06 01:26</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
✅ Veri Güncellendi:  - Sat Mar  7 01:19:10 UTC 2026
</commit_message>
<xml_diff>
--- a/leads_output.xlsx
+++ b/leads_output.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E302"/>
+  <dimension ref="A1:E316"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -9176,6 +9176,412 @@
         </is>
       </c>
     </row>
+    <row r="303">
+      <c r="A303" t="inlineStr">
+        <is>
+          <t>Bağdat Seda Eczanesi</t>
+        </is>
+      </c>
+      <c r="B303" t="inlineStr">
+        <is>
+          <t>
++90 216 356 54 44</t>
+        </is>
+      </c>
+      <c r="C303" t="inlineStr">
+        <is>
+          <t>
+Suadiye, Bağdat Cad. No: 393F D:6, 34740 Kadıköy/İstanbul, Türkiye</t>
+        </is>
+      </c>
+      <c r="D303" t="inlineStr">
+        <is>
+          <t>Kadikoy/Istanbul</t>
+        </is>
+      </c>
+      <c r="E303" t="inlineStr">
+        <is>
+          <t>2026-03-07 01:18</t>
+        </is>
+      </c>
+    </row>
+    <row r="304">
+      <c r="A304" t="inlineStr">
+        <is>
+          <t>Perla Eczanesi</t>
+        </is>
+      </c>
+      <c r="B304" t="inlineStr">
+        <is>
+          <t>
++90 216 372 84 69</t>
+        </is>
+      </c>
+      <c r="C304" t="inlineStr">
+        <is>
+          <t>
+19 Mayıs, Bayar Cd. No: 41-1A, 34736 Kadıköy/İstanbul, Türkiye</t>
+        </is>
+      </c>
+      <c r="D304" t="inlineStr">
+        <is>
+          <t>Kadikoy/Istanbul</t>
+        </is>
+      </c>
+      <c r="E304" t="inlineStr">
+        <is>
+          <t>2026-03-07 01:18</t>
+        </is>
+      </c>
+    </row>
+    <row r="305">
+      <c r="A305" t="inlineStr">
+        <is>
+          <t>KOZA ECZANESİ</t>
+        </is>
+      </c>
+      <c r="B305" t="inlineStr">
+        <is>
+          <t>
++90 216 784 03 04</t>
+        </is>
+      </c>
+      <c r="C305" t="inlineStr">
+        <is>
+          <t>
+Kozyatağı, 19 Mayıs, Begonya Sk. No: 9/A, 34736 Kadıköy/İstanbul, Türkiye</t>
+        </is>
+      </c>
+      <c r="D305" t="inlineStr">
+        <is>
+          <t>Kadikoy/Istanbul</t>
+        </is>
+      </c>
+      <c r="E305" t="inlineStr">
+        <is>
+          <t>2026-03-07 01:18</t>
+        </is>
+      </c>
+    </row>
+    <row r="306">
+      <c r="A306" t="inlineStr">
+        <is>
+          <t>Hilal Eczanesi</t>
+        </is>
+      </c>
+      <c r="B306" t="inlineStr">
+        <is>
+          <t>
++90 216 545 21 12</t>
+        </is>
+      </c>
+      <c r="C306" t="inlineStr">
+        <is>
+          <t>
+Acıbadem, Zeamet Sk. No:4/a, 34718 Kadıköy/İstanbul, Türkiye</t>
+        </is>
+      </c>
+      <c r="D306" t="inlineStr">
+        <is>
+          <t>Kadikoy/Istanbul</t>
+        </is>
+      </c>
+      <c r="E306" t="inlineStr">
+        <is>
+          <t>2026-03-07 01:18</t>
+        </is>
+      </c>
+    </row>
+    <row r="307">
+      <c r="A307" t="inlineStr">
+        <is>
+          <t>Damlataş Eczanesi Göztepe</t>
+        </is>
+      </c>
+      <c r="B307" t="inlineStr">
+        <is>
+          <t>
++90 216 426 07 70</t>
+        </is>
+      </c>
+      <c r="C307" t="inlineStr">
+        <is>
+          <t>
+Göztepe, Tütüncü Mehmet Efendi Cd. No:99, 34730 Kadıköy/İstanbul, Türkiye</t>
+        </is>
+      </c>
+      <c r="D307" t="inlineStr">
+        <is>
+          <t>Kadikoy/Istanbul</t>
+        </is>
+      </c>
+      <c r="E307" t="inlineStr">
+        <is>
+          <t>2026-03-07 01:18</t>
+        </is>
+      </c>
+    </row>
+    <row r="308">
+      <c r="A308" t="inlineStr">
+        <is>
+          <t>GAMZE ECZANESİ</t>
+        </is>
+      </c>
+      <c r="B308" t="inlineStr">
+        <is>
+          <t>
++90 543 209 42 42</t>
+        </is>
+      </c>
+      <c r="C308" t="inlineStr">
+        <is>
+          <t>
+Acıbadem, Acıbadem Cd. No:103a, 34718 Kadıköy/İstanbul, Türkiye</t>
+        </is>
+      </c>
+      <c r="D308" t="inlineStr">
+        <is>
+          <t>Kadikoy/Istanbul</t>
+        </is>
+      </c>
+      <c r="E308" t="inlineStr">
+        <is>
+          <t>2026-03-07 01:18</t>
+        </is>
+      </c>
+    </row>
+    <row r="309">
+      <c r="A309" t="inlineStr">
+        <is>
+          <t>Vanilya Eczanesi</t>
+        </is>
+      </c>
+      <c r="B309" t="inlineStr">
+        <is>
+          <t>
++90 532 546 79 69</t>
+        </is>
+      </c>
+      <c r="C309" t="inlineStr">
+        <is>
+          <t>
+Bostancı Mah, Bağdat Cad, No 454 Edler Apt, Suadiye, 34744 Kadıköy/İstanbul, Türkiye</t>
+        </is>
+      </c>
+      <c r="D309" t="inlineStr">
+        <is>
+          <t>Kadikoy/Istanbul</t>
+        </is>
+      </c>
+      <c r="E309" t="inlineStr">
+        <is>
+          <t>2026-03-07 01:18</t>
+        </is>
+      </c>
+    </row>
+    <row r="310">
+      <c r="A310" t="inlineStr">
+        <is>
+          <t>Bizim Evin Eczanesi</t>
+        </is>
+      </c>
+      <c r="B310" t="inlineStr">
+        <is>
+          <t>
++90 216 566 61 06</t>
+        </is>
+      </c>
+      <c r="C310" t="inlineStr">
+        <is>
+          <t>
+Feneryolu, 34724 Kadıköy/İstanbul, Türkiye</t>
+        </is>
+      </c>
+      <c r="D310" t="inlineStr">
+        <is>
+          <t>Kadikoy/Istanbul</t>
+        </is>
+      </c>
+      <c r="E310" t="inlineStr">
+        <is>
+          <t>2026-03-07 01:18</t>
+        </is>
+      </c>
+    </row>
+    <row r="311">
+      <c r="A311" t="inlineStr">
+        <is>
+          <t>KÖKLÜ ECZANESİ</t>
+        </is>
+      </c>
+      <c r="B311" t="inlineStr">
+        <is>
+          <t>
++90 216 909 40 61</t>
+        </is>
+      </c>
+      <c r="C311" t="inlineStr">
+        <is>
+          <t>
+Bostancı, Kocayol Cd. no:30/a, 34744 Kadıköy/İstanbul, Türkiye</t>
+        </is>
+      </c>
+      <c r="D311" t="inlineStr">
+        <is>
+          <t>Kadikoy/Istanbul</t>
+        </is>
+      </c>
+      <c r="E311" t="inlineStr">
+        <is>
+          <t>2026-03-07 01:18</t>
+        </is>
+      </c>
+    </row>
+    <row r="312">
+      <c r="A312" t="inlineStr">
+        <is>
+          <t>Defne Eczanesi</t>
+        </is>
+      </c>
+      <c r="B312" t="inlineStr">
+        <is>
+          <t>
++90 216 464 58 41</t>
+        </is>
+      </c>
+      <c r="C312" t="inlineStr">
+        <is>
+          <t>
+Suadiye, Emin Ali Paşa Cd. No:11, 34740 Kadıköy/İstanbul, Türkiye</t>
+        </is>
+      </c>
+      <c r="D312" t="inlineStr">
+        <is>
+          <t>Kadikoy/Istanbul</t>
+        </is>
+      </c>
+      <c r="E312" t="inlineStr">
+        <is>
+          <t>2026-03-07 01:18</t>
+        </is>
+      </c>
+    </row>
+    <row r="313">
+      <c r="A313" t="inlineStr">
+        <is>
+          <t>Göztepe Eczanesi</t>
+        </is>
+      </c>
+      <c r="B313" t="inlineStr">
+        <is>
+          <t>
++90 216 566 77 70</t>
+        </is>
+      </c>
+      <c r="C313" t="inlineStr">
+        <is>
+          <t>
+Feneryolu, Fahrettin Kerim Gökay Cd No:142/A, 34724 Kadıköy/İstanbul, Türkiye</t>
+        </is>
+      </c>
+      <c r="D313" t="inlineStr">
+        <is>
+          <t>Kadikoy/Istanbul</t>
+        </is>
+      </c>
+      <c r="E313" t="inlineStr">
+        <is>
+          <t>2026-03-07 01:19</t>
+        </is>
+      </c>
+    </row>
+    <row r="314">
+      <c r="A314" t="inlineStr">
+        <is>
+          <t>Su Eczanesi</t>
+        </is>
+      </c>
+      <c r="B314" t="inlineStr">
+        <is>
+          <t>
++90 216 411 72 28</t>
+        </is>
+      </c>
+      <c r="C314" t="inlineStr">
+        <is>
+          <t>
+Caddebostan, Bağdat Cad. No:288/B, 34728 Kadıköy/İstanbul, Türkiye</t>
+        </is>
+      </c>
+      <c r="D314" t="inlineStr">
+        <is>
+          <t>Kadikoy/Istanbul</t>
+        </is>
+      </c>
+      <c r="E314" t="inlineStr">
+        <is>
+          <t>2026-03-07 01:19</t>
+        </is>
+      </c>
+    </row>
+    <row r="315">
+      <c r="A315" t="inlineStr">
+        <is>
+          <t>Pak Eczanesi</t>
+        </is>
+      </c>
+      <c r="B315" t="inlineStr">
+        <is>
+          <t>
++90 216 339 43 67</t>
+        </is>
+      </c>
+      <c r="C315" t="inlineStr">
+        <is>
+          <t>
+Acıbadem, 34718 Kadıköy/İstanbul, Türkiye</t>
+        </is>
+      </c>
+      <c r="D315" t="inlineStr">
+        <is>
+          <t>Kadikoy/Istanbul</t>
+        </is>
+      </c>
+      <c r="E315" t="inlineStr">
+        <is>
+          <t>2026-03-07 01:19</t>
+        </is>
+      </c>
+    </row>
+    <row r="316">
+      <c r="A316" t="inlineStr">
+        <is>
+          <t>Alioğlu Eczanesi</t>
+        </is>
+      </c>
+      <c r="B316" t="inlineStr">
+        <is>
+          <t>
++90 216 357 47 27</t>
+        </is>
+      </c>
+      <c r="C316" t="inlineStr">
+        <is>
+          <t>
+19 Mayıs, 34736 Kadıköy/İstanbul, Türkiye</t>
+        </is>
+      </c>
+      <c r="D316" t="inlineStr">
+        <is>
+          <t>Kadikoy/Istanbul</t>
+        </is>
+      </c>
+      <c r="E316" t="inlineStr">
+        <is>
+          <t>2026-03-07 01:19</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
✅ Veri Güncellendi:  - Sun Mar  8 01:25:01 UTC 2026
</commit_message>
<xml_diff>
--- a/leads_output.xlsx
+++ b/leads_output.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E316"/>
+  <dimension ref="A1:E318"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -9582,6 +9582,64 @@
         </is>
       </c>
     </row>
+    <row r="317">
+      <c r="A317" t="inlineStr">
+        <is>
+          <t>Akalın Eczanesi</t>
+        </is>
+      </c>
+      <c r="B317" t="inlineStr">
+        <is>
+          <t>
++90 216 566 03 30</t>
+        </is>
+      </c>
+      <c r="C317" t="inlineStr">
+        <is>
+          <t>
+Merdivenköy, Şair Arşi Cd. No:7, 34732 Kadıköy/İstanbul, Türkiye</t>
+        </is>
+      </c>
+      <c r="D317" t="inlineStr">
+        <is>
+          <t>Kadikoy/Istanbul</t>
+        </is>
+      </c>
+      <c r="E317" t="inlineStr">
+        <is>
+          <t>2026-03-08 01:24</t>
+        </is>
+      </c>
+    </row>
+    <row r="318">
+      <c r="A318" t="inlineStr">
+        <is>
+          <t>Eczane Salt</t>
+        </is>
+      </c>
+      <c r="B318" t="inlineStr">
+        <is>
+          <t>
++90 216 999 56 70</t>
+        </is>
+      </c>
+      <c r="C318" t="inlineStr">
+        <is>
+          <t>
+Brooklyn Park, Merdivenköy, Seyhan Sk. No: 13 A1 Blok, 34732 Kadıköy/İstanbul, Türkiye</t>
+        </is>
+      </c>
+      <c r="D318" t="inlineStr">
+        <is>
+          <t>Kadikoy/Istanbul</t>
+        </is>
+      </c>
+      <c r="E318" t="inlineStr">
+        <is>
+          <t>2026-03-08 01:25</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
✅ Veri Güncellendi:  - Tue Mar 10 01:19:25 UTC 2026
</commit_message>
<xml_diff>
--- a/leads_output.xlsx
+++ b/leads_output.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E318"/>
+  <dimension ref="A1:E322"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -9640,6 +9640,122 @@
         </is>
       </c>
     </row>
+    <row r="319">
+      <c r="A319" t="inlineStr">
+        <is>
+          <t>Ethem Efendi Eczanesi</t>
+        </is>
+      </c>
+      <c r="B319" t="inlineStr">
+        <is>
+          <t>
++90 216 476 00 34</t>
+        </is>
+      </c>
+      <c r="C319" t="inlineStr">
+        <is>
+          <t>
+Erenköy, Ethemefendi Caddesi No:63 D:1A, 34738 Kadıköy/İstanbul, Türkiye</t>
+        </is>
+      </c>
+      <c r="D319" t="inlineStr">
+        <is>
+          <t>Kadikoy/Istanbul</t>
+        </is>
+      </c>
+      <c r="E319" t="inlineStr">
+        <is>
+          <t>2026-03-10 01:19</t>
+        </is>
+      </c>
+    </row>
+    <row r="320">
+      <c r="A320" t="inlineStr">
+        <is>
+          <t>Suadiye Banu Eczanesi</t>
+        </is>
+      </c>
+      <c r="B320" t="inlineStr">
+        <is>
+          <t>
++90 530 664 61 41</t>
+        </is>
+      </c>
+      <c r="C320" t="inlineStr">
+        <is>
+          <t>
+Suadiye, Ayşeçavuş Cd No: 35B, 34734 Kadıköy/İstanbul, Türkiye</t>
+        </is>
+      </c>
+      <c r="D320" t="inlineStr">
+        <is>
+          <t>Kadikoy/Istanbul</t>
+        </is>
+      </c>
+      <c r="E320" t="inlineStr">
+        <is>
+          <t>2026-03-10 01:19</t>
+        </is>
+      </c>
+    </row>
+    <row r="321">
+      <c r="A321" t="inlineStr">
+        <is>
+          <t>Nur Karataş Eczanesi</t>
+        </is>
+      </c>
+      <c r="B321" t="inlineStr">
+        <is>
+          <t>
++90 501 133 06 87</t>
+        </is>
+      </c>
+      <c r="C321" t="inlineStr">
+        <is>
+          <t>
+Caferağa, Moda Cd. No:106A, 34710 Kadıköy/İstanbul, Türkiye</t>
+        </is>
+      </c>
+      <c r="D321" t="inlineStr">
+        <is>
+          <t>Kadikoy/Istanbul</t>
+        </is>
+      </c>
+      <c r="E321" t="inlineStr">
+        <is>
+          <t>2026-03-10 01:19</t>
+        </is>
+      </c>
+    </row>
+    <row r="322">
+      <c r="A322" t="inlineStr">
+        <is>
+          <t>Eczane İrem Özdoğan</t>
+        </is>
+      </c>
+      <c r="B322" t="inlineStr">
+        <is>
+          <t>
++90 216 565 19 50</t>
+        </is>
+      </c>
+      <c r="C322" t="inlineStr">
+        <is>
+          <t>
+Kadıköy (GATE OTEL YANI-TÜRK TELEKOM SOKAĞI, Göztepe mahallesi, Göztepe, Çimenzar Sk. No:36/A, 34730 Kadıköy/İstanbul, Türkiye</t>
+        </is>
+      </c>
+      <c r="D322" t="inlineStr">
+        <is>
+          <t>Kadikoy/Istanbul</t>
+        </is>
+      </c>
+      <c r="E322" t="inlineStr">
+        <is>
+          <t>2026-03-10 01:19</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
✅ Veri Güncellendi:  - Wed Mar 11 01:19:39 UTC 2026
</commit_message>
<xml_diff>
--- a/leads_output.xlsx
+++ b/leads_output.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E322"/>
+  <dimension ref="A1:E326"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -9756,6 +9756,122 @@
         </is>
       </c>
     </row>
+    <row r="323">
+      <c r="A323" t="inlineStr">
+        <is>
+          <t>SAKURA ECZANESİ</t>
+        </is>
+      </c>
+      <c r="B323" t="inlineStr">
+        <is>
+          <t>
++90 532 430 02 59</t>
+        </is>
+      </c>
+      <c r="C323" t="inlineStr">
+        <is>
+          <t>
+Osmanağa, Başçavuş Sk. No:8/A, 34714 Kadıköy/İstanbul, Türkiye</t>
+        </is>
+      </c>
+      <c r="D323" t="inlineStr">
+        <is>
+          <t>Kadikoy/Istanbul</t>
+        </is>
+      </c>
+      <c r="E323" t="inlineStr">
+        <is>
+          <t>2026-03-11 01:19</t>
+        </is>
+      </c>
+    </row>
+    <row r="324">
+      <c r="A324" t="inlineStr">
+        <is>
+          <t>Feyzan Eczanesi</t>
+        </is>
+      </c>
+      <c r="B324" t="inlineStr">
+        <is>
+          <t>
++90 216 345 37 74</t>
+        </is>
+      </c>
+      <c r="C324" t="inlineStr">
+        <is>
+          <t>
+Feneryolu Mah. Fahrettin Kerim Gökay Cad. Tuğrul Apt, No:102/C, 34724 Kadıköy/İstanbul, Türkiye</t>
+        </is>
+      </c>
+      <c r="D324" t="inlineStr">
+        <is>
+          <t>Kadikoy/Istanbul</t>
+        </is>
+      </c>
+      <c r="E324" t="inlineStr">
+        <is>
+          <t>2026-03-11 01:19</t>
+        </is>
+      </c>
+    </row>
+    <row r="325">
+      <c r="A325" t="inlineStr">
+        <is>
+          <t>Cadde Eczanesi</t>
+        </is>
+      </c>
+      <c r="B325" t="inlineStr">
+        <is>
+          <t>
++90 216 386 64 44</t>
+        </is>
+      </c>
+      <c r="C325" t="inlineStr">
+        <is>
+          <t>
+Suadiye mahallesi vapur yolu sokak özlü apartmanı, No 2/B, 34740 Kadıköy/İstanbul, Türkiye</t>
+        </is>
+      </c>
+      <c r="D325" t="inlineStr">
+        <is>
+          <t>Kadikoy/Istanbul</t>
+        </is>
+      </c>
+      <c r="E325" t="inlineStr">
+        <is>
+          <t>2026-03-11 01:19</t>
+        </is>
+      </c>
+    </row>
+    <row r="326">
+      <c r="A326" t="inlineStr">
+        <is>
+          <t>Eczane İskele Huzur</t>
+        </is>
+      </c>
+      <c r="B326" t="inlineStr">
+        <is>
+          <t>
++90 216 346 54 09</t>
+        </is>
+      </c>
+      <c r="C326" t="inlineStr">
+        <is>
+          <t>
+Caferağa, Albay Faik Sözdener Cd. No:7 D:B, 34710 Kadıköy/İstanbul, Türkiye</t>
+        </is>
+      </c>
+      <c r="D326" t="inlineStr">
+        <is>
+          <t>Kadikoy/Istanbul</t>
+        </is>
+      </c>
+      <c r="E326" t="inlineStr">
+        <is>
+          <t>2026-03-11 01:19</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
✅ Veri Güncellendi:  - Thu Mar 12 01:20:16 UTC 2026
</commit_message>
<xml_diff>
--- a/leads_output.xlsx
+++ b/leads_output.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E326"/>
+  <dimension ref="A1:E339"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -9872,6 +9872,383 @@
         </is>
       </c>
     </row>
+    <row r="327">
+      <c r="A327" t="inlineStr">
+        <is>
+          <t>Melike Eczanesi</t>
+        </is>
+      </c>
+      <c r="B327" t="inlineStr">
+        <is>
+          <t>
++90 216 459 41 14</t>
+        </is>
+      </c>
+      <c r="C327" t="inlineStr">
+        <is>
+          <t>
+284, Feyzullah, Bağdat Cad. Yüzevler, 34843 Maltepe/İstanbul, Türkiye</t>
+        </is>
+      </c>
+      <c r="D327" t="inlineStr">
+        <is>
+          <t>Kadikoy/Istanbul</t>
+        </is>
+      </c>
+      <c r="E327" t="inlineStr">
+        <is>
+          <t>2026-03-12 01:19</t>
+        </is>
+      </c>
+    </row>
+    <row r="328">
+      <c r="A328" t="inlineStr">
+        <is>
+          <t>Tanyer Eczanesi</t>
+        </is>
+      </c>
+      <c r="B328" t="inlineStr">
+        <is>
+          <t>
++90 216 355 52 29</t>
+        </is>
+      </c>
+      <c r="C328" t="inlineStr">
+        <is>
+          <t>
+Selamiçeşme, Bağdat Cad. No: 185/A, 34730 Kadıköy/İstanbul, Türkiye</t>
+        </is>
+      </c>
+      <c r="D328" t="inlineStr">
+        <is>
+          <t>Kadikoy/Istanbul</t>
+        </is>
+      </c>
+      <c r="E328" t="inlineStr">
+        <is>
+          <t>2026-03-12 01:19</t>
+        </is>
+      </c>
+    </row>
+    <row r="329">
+      <c r="A329" t="inlineStr">
+        <is>
+          <t>Eczane Yaşam</t>
+        </is>
+      </c>
+      <c r="B329" t="inlineStr">
+        <is>
+          <t>
++90 216 345 71 31</t>
+        </is>
+      </c>
+      <c r="C329" t="inlineStr">
+        <is>
+          <t>
+Eğitim, Nahitbey Sok. No:13/1, 34000 Kadıköy/İstanbul, Türkiye</t>
+        </is>
+      </c>
+      <c r="D329" t="inlineStr">
+        <is>
+          <t>Kadikoy/Istanbul</t>
+        </is>
+      </c>
+      <c r="E329" t="inlineStr">
+        <is>
+          <t>2026-03-12 01:19</t>
+        </is>
+      </c>
+    </row>
+    <row r="330">
+      <c r="A330" t="inlineStr">
+        <is>
+          <t>Şua Eczanesi/ Şua Pharmacy</t>
+        </is>
+      </c>
+      <c r="B330" t="inlineStr">
+        <is>
+          <t>
++90 531 221 83 87</t>
+        </is>
+      </c>
+      <c r="C330" t="inlineStr">
+        <is>
+          <t>
+Şua Elite Concept, No:2F Ticari Alan:9, Fikirtepe, Barış Sk. A Blok, 34720 Kadıköy/İstanbul, Türkiye</t>
+        </is>
+      </c>
+      <c r="D330" t="inlineStr">
+        <is>
+          <t>Kadikoy/Istanbul</t>
+        </is>
+      </c>
+      <c r="E330" t="inlineStr">
+        <is>
+          <t>2026-03-12 01:19</t>
+        </is>
+      </c>
+    </row>
+    <row r="331">
+      <c r="A331" t="inlineStr">
+        <is>
+          <t>Rıhtım Eczane Ve Optik</t>
+        </is>
+      </c>
+      <c r="B331" t="inlineStr">
+        <is>
+          <t>
++90 216 337 31 38</t>
+        </is>
+      </c>
+      <c r="C331" t="inlineStr">
+        <is>
+          <t>
+Osmanağa, Söğütlüçeşme Cad. No:39, 34714 Kadıköy/İstanbul, Türkiye</t>
+        </is>
+      </c>
+      <c r="D331" t="inlineStr">
+        <is>
+          <t>Kadikoy/Istanbul</t>
+        </is>
+      </c>
+      <c r="E331" t="inlineStr">
+        <is>
+          <t>2026-03-12 01:19</t>
+        </is>
+      </c>
+    </row>
+    <row r="332">
+      <c r="A332" t="inlineStr">
+        <is>
+          <t>Ürün Eczanesi</t>
+        </is>
+      </c>
+      <c r="B332" t="inlineStr">
+        <is>
+          <t>
++90 532 226 50 68</t>
+        </is>
+      </c>
+      <c r="C332" t="inlineStr">
+        <is>
+          <t>
+Bostancı, Camevler Sk. No:9 D:C, 34744 Kadıköy/İstanbul, Türkiye</t>
+        </is>
+      </c>
+      <c r="D332" t="inlineStr">
+        <is>
+          <t>Kadikoy/Istanbul</t>
+        </is>
+      </c>
+      <c r="E332" t="inlineStr">
+        <is>
+          <t>2026-03-12 01:19</t>
+        </is>
+      </c>
+    </row>
+    <row r="333">
+      <c r="A333" t="inlineStr">
+        <is>
+          <t>Orkun Eczanesi (English speaking pharmacy) Apotheke, Pharmacy</t>
+        </is>
+      </c>
+      <c r="B333" t="inlineStr">
+        <is>
+          <t>
++90 216 464 76 48</t>
+        </is>
+      </c>
+      <c r="C333" t="inlineStr">
+        <is>
+          <t>
+Kozyatağı, Hilmi Paşa Sk No:42 D:E, 34742 Kadıköy/İstanbul, Türkiye</t>
+        </is>
+      </c>
+      <c r="D333" t="inlineStr">
+        <is>
+          <t>Kadikoy/Istanbul</t>
+        </is>
+      </c>
+      <c r="E333" t="inlineStr">
+        <is>
+          <t>2026-03-12 01:19</t>
+        </is>
+      </c>
+    </row>
+    <row r="334">
+      <c r="A334" t="inlineStr">
+        <is>
+          <t>İlçim Eczanesi</t>
+        </is>
+      </c>
+      <c r="B334" t="inlineStr">
+        <is>
+          <t>
++90 216 368 99 98</t>
+        </is>
+      </c>
+      <c r="C334" t="inlineStr">
+        <is>
+          <t>
+Fenerbahçe, Dr. Faruk Ayanoğlu Cd. No:2, 34726 Kadıköy/İstanbul, Türkiye</t>
+        </is>
+      </c>
+      <c r="D334" t="inlineStr">
+        <is>
+          <t>Kadikoy/Istanbul</t>
+        </is>
+      </c>
+      <c r="E334" t="inlineStr">
+        <is>
+          <t>2026-03-12 01:20</t>
+        </is>
+      </c>
+    </row>
+    <row r="335">
+      <c r="A335" t="inlineStr">
+        <is>
+          <t>İrem Eczanesi</t>
+        </is>
+      </c>
+      <c r="B335" t="inlineStr">
+        <is>
+          <t>
++90 216 463 50 51</t>
+        </is>
+      </c>
+      <c r="C335" t="inlineStr">
+        <is>
+          <t>
+Kozyatağı, Şemsettin Günaltay Cd. NO:32-34/A, 34742 Kadıköy/İstanbul, Türkiye</t>
+        </is>
+      </c>
+      <c r="D335" t="inlineStr">
+        <is>
+          <t>Kadikoy/Istanbul</t>
+        </is>
+      </c>
+      <c r="E335" t="inlineStr">
+        <is>
+          <t>2026-03-12 01:20</t>
+        </is>
+      </c>
+    </row>
+    <row r="336">
+      <c r="A336" t="inlineStr">
+        <is>
+          <t>Beytül Eczanesi</t>
+        </is>
+      </c>
+      <c r="B336" t="inlineStr">
+        <is>
+          <t>
++90 216 428 54 50</t>
+        </is>
+      </c>
+      <c r="C336" t="inlineStr">
+        <is>
+          <t>
+Acıbadem, Sokullu Sokağı no:4/A, 34718 Kadıköy/İstanbul, Türkiye</t>
+        </is>
+      </c>
+      <c r="D336" t="inlineStr">
+        <is>
+          <t>Kadikoy/Istanbul</t>
+        </is>
+      </c>
+      <c r="E336" t="inlineStr">
+        <is>
+          <t>2026-03-12 01:20</t>
+        </is>
+      </c>
+    </row>
+    <row r="337">
+      <c r="A337" t="inlineStr">
+        <is>
+          <t>Kamelya Eczanesi</t>
+        </is>
+      </c>
+      <c r="B337" t="inlineStr">
+        <is>
+          <t>
++90 216 428 54 50</t>
+        </is>
+      </c>
+      <c r="C337" t="inlineStr">
+        <is>
+          <t>
+Acıbadem, Sokullu Sokağı no:4/A, 34718 Kadıköy/İstanbul, Türkiye</t>
+        </is>
+      </c>
+      <c r="D337" t="inlineStr">
+        <is>
+          <t>Kadikoy/Istanbul</t>
+        </is>
+      </c>
+      <c r="E337" t="inlineStr">
+        <is>
+          <t>2026-03-12 01:20</t>
+        </is>
+      </c>
+    </row>
+    <row r="338">
+      <c r="A338" t="inlineStr">
+        <is>
+          <t>Gaye Eczanesi</t>
+        </is>
+      </c>
+      <c r="B338" t="inlineStr">
+        <is>
+          <t>
++90 216 360 64 45</t>
+        </is>
+      </c>
+      <c r="C338" t="inlineStr">
+        <is>
+          <t>
+Caddebostan, Ömer Paşa Sk. 12/1, 34728 Kadıköy/İstanbul, Türkiye</t>
+        </is>
+      </c>
+      <c r="D338" t="inlineStr">
+        <is>
+          <t>Kadikoy/Istanbul</t>
+        </is>
+      </c>
+      <c r="E338" t="inlineStr">
+        <is>
+          <t>2026-03-12 01:20</t>
+        </is>
+      </c>
+    </row>
+    <row r="339">
+      <c r="A339" t="inlineStr">
+        <is>
+          <t>Esat Eczanesi</t>
+        </is>
+      </c>
+      <c r="B339" t="inlineStr">
+        <is>
+          <t>
++90 216 325 25 35</t>
+        </is>
+      </c>
+      <c r="C339" t="inlineStr">
+        <is>
+          <t>
+Koşuyolu, Tekin Sk. 7C D:B, 34718 Kadıköy/İstanbul, Türkiye</t>
+        </is>
+      </c>
+      <c r="D339" t="inlineStr">
+        <is>
+          <t>Kadikoy/Istanbul</t>
+        </is>
+      </c>
+      <c r="E339" t="inlineStr">
+        <is>
+          <t>2026-03-12 01:20</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
✅ Veri Güncellendi:  - Fri Mar 13 01:23:19 UTC 2026
</commit_message>
<xml_diff>
--- a/leads_output.xlsx
+++ b/leads_output.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E339"/>
+  <dimension ref="A1:E341"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -10249,6 +10249,64 @@
         </is>
       </c>
     </row>
+    <row r="340">
+      <c r="A340" t="inlineStr">
+        <is>
+          <t>Terece Eczanesi</t>
+        </is>
+      </c>
+      <c r="B340" t="inlineStr">
+        <is>
+          <t>
++90 216 360 50 59</t>
+        </is>
+      </c>
+      <c r="C340" t="inlineStr">
+        <is>
+          <t>
+Caddebostan, Bağdat Cad. No:350/A, 34728 Kadıköy/İstanbul, Türkiye</t>
+        </is>
+      </c>
+      <c r="D340" t="inlineStr">
+        <is>
+          <t>Kadikoy/Istanbul</t>
+        </is>
+      </c>
+      <c r="E340" t="inlineStr">
+        <is>
+          <t>2026-03-13 01:23</t>
+        </is>
+      </c>
+    </row>
+    <row r="341">
+      <c r="A341" t="inlineStr">
+        <is>
+          <t>Melis Hanlı Eczanesi</t>
+        </is>
+      </c>
+      <c r="B341" t="inlineStr">
+        <is>
+          <t>
++90 551 591 77 97</t>
+        </is>
+      </c>
+      <c r="C341" t="inlineStr">
+        <is>
+          <t>
+Erenköy, Ömer Paşa Sk. No:54A, 34738 Kadıköy/İstanbul, Türkiye</t>
+        </is>
+      </c>
+      <c r="D341" t="inlineStr">
+        <is>
+          <t>Kadikoy/Istanbul</t>
+        </is>
+      </c>
+      <c r="E341" t="inlineStr">
+        <is>
+          <t>2026-03-13 01:23</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
✅ Veri Güncellendi:  - Sat Mar 14 01:21:45 UTC 2026
</commit_message>
<xml_diff>
--- a/leads_output.xlsx
+++ b/leads_output.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E341"/>
+  <dimension ref="A1:E349"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -10307,6 +10307,238 @@
         </is>
       </c>
     </row>
+    <row r="342">
+      <c r="A342" t="inlineStr">
+        <is>
+          <t>Eczane Cankız</t>
+        </is>
+      </c>
+      <c r="B342" t="inlineStr">
+        <is>
+          <t>
++90 216 803 73 43</t>
+        </is>
+      </c>
+      <c r="C342" t="inlineStr">
+        <is>
+          <t>
+Erenköy, Erenköy İstasyon Cd. No:35C, 34738 Kadıköy/İstanbul, Türkiye</t>
+        </is>
+      </c>
+      <c r="D342" t="inlineStr">
+        <is>
+          <t>Kadikoy/Istanbul</t>
+        </is>
+      </c>
+      <c r="E342" t="inlineStr">
+        <is>
+          <t>2026-03-14 01:21</t>
+        </is>
+      </c>
+    </row>
+    <row r="343">
+      <c r="A343" t="inlineStr">
+        <is>
+          <t>Eczane Dumlupınar</t>
+        </is>
+      </c>
+      <c r="B343" t="inlineStr">
+        <is>
+          <t>
++90 216 565 07 06</t>
+        </is>
+      </c>
+      <c r="C343" t="inlineStr">
+        <is>
+          <t>
+Dumlupınar, Mektep Sk. No:11, 34720 Kadıköy/İstanbul, Türkiye</t>
+        </is>
+      </c>
+      <c r="D343" t="inlineStr">
+        <is>
+          <t>Kadikoy/Istanbul</t>
+        </is>
+      </c>
+      <c r="E343" t="inlineStr">
+        <is>
+          <t>2026-03-14 01:21</t>
+        </is>
+      </c>
+    </row>
+    <row r="344">
+      <c r="A344" t="inlineStr">
+        <is>
+          <t>Eczane Aylin</t>
+        </is>
+      </c>
+      <c r="B344" t="inlineStr">
+        <is>
+          <t>
++90 216 385 36 78</t>
+        </is>
+      </c>
+      <c r="C344" t="inlineStr">
+        <is>
+          <t>
+Sahrayı Cedit, Cami Sk., 34734 Kadıköy/İstanbul, Türkiye</t>
+        </is>
+      </c>
+      <c r="D344" t="inlineStr">
+        <is>
+          <t>Kadikoy/Istanbul</t>
+        </is>
+      </c>
+      <c r="E344" t="inlineStr">
+        <is>
+          <t>2026-03-14 01:21</t>
+        </is>
+      </c>
+    </row>
+    <row r="345">
+      <c r="A345" t="inlineStr">
+        <is>
+          <t>Timsal Eczane</t>
+        </is>
+      </c>
+      <c r="B345" t="inlineStr">
+        <is>
+          <t>
++90 216 445 21 25</t>
+        </is>
+      </c>
+      <c r="C345" t="inlineStr">
+        <is>
+          <t>
+Suadiye, Kaptan Arif Sok. No:44, 34740 Kadıköy/İstanbul, Türkiye</t>
+        </is>
+      </c>
+      <c r="D345" t="inlineStr">
+        <is>
+          <t>Kadikoy/Istanbul</t>
+        </is>
+      </c>
+      <c r="E345" t="inlineStr">
+        <is>
+          <t>2026-03-14 01:21</t>
+        </is>
+      </c>
+    </row>
+    <row r="346">
+      <c r="A346" t="inlineStr">
+        <is>
+          <t>SEVDE ECZANESİ</t>
+        </is>
+      </c>
+      <c r="B346" t="inlineStr">
+        <is>
+          <t>
++90 533 363 45 93</t>
+        </is>
+      </c>
+      <c r="C346" t="inlineStr">
+        <is>
+          <t>
+Bostancı, Yalı Yolu Sk. No:27/A, 34744 Kadıköy/İstanbul, Türkiye</t>
+        </is>
+      </c>
+      <c r="D346" t="inlineStr">
+        <is>
+          <t>Kadikoy/Istanbul</t>
+        </is>
+      </c>
+      <c r="E346" t="inlineStr">
+        <is>
+          <t>2026-03-14 01:21</t>
+        </is>
+      </c>
+    </row>
+    <row r="347">
+      <c r="A347" t="inlineStr">
+        <is>
+          <t>AYDIN ECZANESİ</t>
+        </is>
+      </c>
+      <c r="B347" t="inlineStr">
+        <is>
+          <t>
++90 216 766 38 39</t>
+        </is>
+      </c>
+      <c r="C347" t="inlineStr">
+        <is>
+          <t>
+Erenköy, Çamlıköşk Sk. No:5/A, 34738 Kadıköy/İstanbul, Türkiye</t>
+        </is>
+      </c>
+      <c r="D347" t="inlineStr">
+        <is>
+          <t>Kadikoy/Istanbul</t>
+        </is>
+      </c>
+      <c r="E347" t="inlineStr">
+        <is>
+          <t>2026-03-14 01:21</t>
+        </is>
+      </c>
+    </row>
+    <row r="348">
+      <c r="A348" t="inlineStr">
+        <is>
+          <t>Cansu Eczanesi</t>
+        </is>
+      </c>
+      <c r="B348" t="inlineStr">
+        <is>
+          <t>
++90 216 348 78 14</t>
+        </is>
+      </c>
+      <c r="C348" t="inlineStr">
+        <is>
+          <t>
+Hekimoğlu Apt, Zühtüpaşa, Cemre Sok. No:1A, 34724 Kadıköy/İstanbul, Türkiye</t>
+        </is>
+      </c>
+      <c r="D348" t="inlineStr">
+        <is>
+          <t>Kadikoy/Istanbul</t>
+        </is>
+      </c>
+      <c r="E348" t="inlineStr">
+        <is>
+          <t>2026-03-14 01:21</t>
+        </is>
+      </c>
+    </row>
+    <row r="349">
+      <c r="A349" t="inlineStr">
+        <is>
+          <t>Eczane Yalvaç</t>
+        </is>
+      </c>
+      <c r="B349" t="inlineStr">
+        <is>
+          <t>
++90 216 411 36 38</t>
+        </is>
+      </c>
+      <c r="C349" t="inlineStr">
+        <is>
+          <t>
+Dostlar apt, Erenköy, Ülke Sk. 15/A, 34738 Kadıköy/İstanbul, Türkiye</t>
+        </is>
+      </c>
+      <c r="D349" t="inlineStr">
+        <is>
+          <t>Kadikoy/Istanbul</t>
+        </is>
+      </c>
+      <c r="E349" t="inlineStr">
+        <is>
+          <t>2026-03-14 01:21</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
✅ Veri Güncellendi:  - Sun Mar 15 01:46:19 UTC 2026
</commit_message>
<xml_diff>
--- a/leads_output.xlsx
+++ b/leads_output.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E349"/>
+  <dimension ref="A1:E351"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -10539,6 +10539,64 @@
         </is>
       </c>
     </row>
+    <row r="350">
+      <c r="A350" t="inlineStr">
+        <is>
+          <t>Batuhan Eczane</t>
+        </is>
+      </c>
+      <c r="B350" t="inlineStr">
+        <is>
+          <t>
++90 216 410 23 01</t>
+        </is>
+      </c>
+      <c r="C350" t="inlineStr">
+        <is>
+          <t>
+Kozyatağı, Bayar Caddesi, Değirmen Sokak Derya Sitesi 6/A B-1 Blok, 34742 Kadıköy/İstanbul, Türkiye</t>
+        </is>
+      </c>
+      <c r="D350" t="inlineStr">
+        <is>
+          <t>Kadikoy/Istanbul</t>
+        </is>
+      </c>
+      <c r="E350" t="inlineStr">
+        <is>
+          <t>2026-03-15 01:46</t>
+        </is>
+      </c>
+    </row>
+    <row r="351">
+      <c r="A351" t="inlineStr">
+        <is>
+          <t>Eczane Vital</t>
+        </is>
+      </c>
+      <c r="B351" t="inlineStr">
+        <is>
+          <t>
++90 216 372 23 29</t>
+        </is>
+      </c>
+      <c r="C351" t="inlineStr">
+        <is>
+          <t>
+Suadiye, Suadiye Camii Sk. 18/A, 34740 Kadıköy/İstanbul, Türkiye</t>
+        </is>
+      </c>
+      <c r="D351" t="inlineStr">
+        <is>
+          <t>Kadikoy/Istanbul</t>
+        </is>
+      </c>
+      <c r="E351" t="inlineStr">
+        <is>
+          <t>2026-03-15 01:46</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
✅ Veri Güncellendi:  - Mon Mar 16 01:48:12 UTC 2026
</commit_message>
<xml_diff>
--- a/leads_output.xlsx
+++ b/leads_output.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E351"/>
+  <dimension ref="A1:E354"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -10597,6 +10597,93 @@
         </is>
       </c>
     </row>
+    <row r="352">
+      <c r="A352" t="inlineStr">
+        <is>
+          <t>KALE ECZANESİ</t>
+        </is>
+      </c>
+      <c r="B352" t="inlineStr">
+        <is>
+          <t>
++90 546 455 46 68</t>
+        </is>
+      </c>
+      <c r="C352" t="inlineStr">
+        <is>
+          <t>
+Merdivenköy, Ressam Salih Erimez Cad No:36B, 34732 Kadıköy/İstanbul, Türkiye</t>
+        </is>
+      </c>
+      <c r="D352" t="inlineStr">
+        <is>
+          <t>Kadikoy/Istanbul</t>
+        </is>
+      </c>
+      <c r="E352" t="inlineStr">
+        <is>
+          <t>2026-03-16 01:48</t>
+        </is>
+      </c>
+    </row>
+    <row r="353">
+      <c r="A353" t="inlineStr">
+        <is>
+          <t>ECZANE REYHAN</t>
+        </is>
+      </c>
+      <c r="B353" t="inlineStr">
+        <is>
+          <t>
++90 216 362 57 05</t>
+        </is>
+      </c>
+      <c r="C353" t="inlineStr">
+        <is>
+          <t>
+Bostancı, Bostan Tariki Sk. 8/A, 34744 Kadıköy/İstanbul, Türkiye</t>
+        </is>
+      </c>
+      <c r="D353" t="inlineStr">
+        <is>
+          <t>Kadikoy/Istanbul</t>
+        </is>
+      </c>
+      <c r="E353" t="inlineStr">
+        <is>
+          <t>2026-03-16 01:48</t>
+        </is>
+      </c>
+    </row>
+    <row r="354">
+      <c r="A354" t="inlineStr">
+        <is>
+          <t>Duru Eczanesi</t>
+        </is>
+      </c>
+      <c r="B354" t="inlineStr">
+        <is>
+          <t>
++90 216 519 59 55</t>
+        </is>
+      </c>
+      <c r="C354" t="inlineStr">
+        <is>
+          <t>
+Erenköy, Kantarcı Rıza Sk. No:3, 34728 Kadıköy/İstanbul, Türkiye</t>
+        </is>
+      </c>
+      <c r="D354" t="inlineStr">
+        <is>
+          <t>Kadikoy/Istanbul</t>
+        </is>
+      </c>
+      <c r="E354" t="inlineStr">
+        <is>
+          <t>2026-03-16 01:48</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
✅ Veri Güncellendi:  - Tue Mar 17 01:25:40 UTC 2026
</commit_message>
<xml_diff>
--- a/leads_output.xlsx
+++ b/leads_output.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E354"/>
+  <dimension ref="A1:E355"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -10684,6 +10684,35 @@
         </is>
       </c>
     </row>
+    <row r="355">
+      <c r="A355" t="inlineStr">
+        <is>
+          <t>Koşuyolu Niş Eczanesi</t>
+        </is>
+      </c>
+      <c r="B355" t="inlineStr">
+        <is>
+          <t>
++90 216 340 88 06</t>
+        </is>
+      </c>
+      <c r="C355" t="inlineStr">
+        <is>
+          <t>
+Koşuyolu, Koşuyolu Cd. No: 109/A, 34718 Kadıköy/İstanbul, Türkiye</t>
+        </is>
+      </c>
+      <c r="D355" t="inlineStr">
+        <is>
+          <t>Kadikoy/Istanbul</t>
+        </is>
+      </c>
+      <c r="E355" t="inlineStr">
+        <is>
+          <t>2026-03-17 01:25</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
✅ Veri Güncellendi:  - Wed Mar 18 01:28:34 UTC 2026
</commit_message>
<xml_diff>
--- a/leads_output.xlsx
+++ b/leads_output.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E355"/>
+  <dimension ref="A1:E356"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -10713,6 +10713,35 @@
         </is>
       </c>
     </row>
+    <row r="356">
+      <c r="A356" t="inlineStr">
+        <is>
+          <t>Eczane Yenidilek</t>
+        </is>
+      </c>
+      <c r="B356" t="inlineStr">
+        <is>
+          <t>
++90 216 362 06 46</t>
+        </is>
+      </c>
+      <c r="C356" t="inlineStr">
+        <is>
+          <t>
+Kozyatağı, Okul Sk. No:3, 34742 Kadıköy/İstanbul, Türkiye</t>
+        </is>
+      </c>
+      <c r="D356" t="inlineStr">
+        <is>
+          <t>Kadikoy/Istanbul</t>
+        </is>
+      </c>
+      <c r="E356" t="inlineStr">
+        <is>
+          <t>2026-03-18 01:28</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
✅ Veri Güncellendi:  - Thu Mar 19 01:29:04 UTC 2026
</commit_message>
<xml_diff>
--- a/leads_output.xlsx
+++ b/leads_output.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E356"/>
+  <dimension ref="A1:E358"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -10742,6 +10742,64 @@
         </is>
       </c>
     </row>
+    <row r="357">
+      <c r="A357" t="inlineStr">
+        <is>
+          <t>ANKA ECZANESİ ACIBADEM</t>
+        </is>
+      </c>
+      <c r="B357" t="inlineStr">
+        <is>
+          <t>
++90 216 771 50 40</t>
+        </is>
+      </c>
+      <c r="C357" t="inlineStr">
+        <is>
+          <t>
+Acıbadem, Acıbadem Cd. No:76, 34718 Kadıköy/İstanbul, Türkiye</t>
+        </is>
+      </c>
+      <c r="D357" t="inlineStr">
+        <is>
+          <t>Kadikoy/Istanbul</t>
+        </is>
+      </c>
+      <c r="E357" t="inlineStr">
+        <is>
+          <t>2026-03-19 01:29</t>
+        </is>
+      </c>
+    </row>
+    <row r="358">
+      <c r="A358" t="inlineStr">
+        <is>
+          <t>Eczane Cansu Kahraman</t>
+        </is>
+      </c>
+      <c r="B358" t="inlineStr">
+        <is>
+          <t>
++90 216 414 54 44</t>
+        </is>
+      </c>
+      <c r="C358" t="inlineStr">
+        <is>
+          <t>
+Osmanağa, Gen. Asım Gündüz Caddesi No:44/A, 34714 Kadıköy/İstanbul, Türkiye</t>
+        </is>
+      </c>
+      <c r="D358" t="inlineStr">
+        <is>
+          <t>Kadikoy/Istanbul</t>
+        </is>
+      </c>
+      <c r="E358" t="inlineStr">
+        <is>
+          <t>2026-03-19 01:29</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
✅ Veri Güncellendi:  - Sun Mar 22 01:28:35 UTC 2026
</commit_message>
<xml_diff>
--- a/leads_output.xlsx
+++ b/leads_output.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E358"/>
+  <dimension ref="A1:E359"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -10800,6 +10800,35 @@
         </is>
       </c>
     </row>
+    <row r="359">
+      <c r="A359" t="inlineStr">
+        <is>
+          <t>KOZYATAĞI GÜL ECZANESİ</t>
+        </is>
+      </c>
+      <c r="B359" t="inlineStr">
+        <is>
+          <t>
++90 501 082 84 80</t>
+        </is>
+      </c>
+      <c r="C359" t="inlineStr">
+        <is>
+          <t>
+Fikirtepe Mah. Mandıra Cad. Mandarins No:11H, 34720 Kadıköy/İstanbul, Türkiye</t>
+        </is>
+      </c>
+      <c r="D359" t="inlineStr">
+        <is>
+          <t>Kadikoy/Istanbul</t>
+        </is>
+      </c>
+      <c r="E359" t="inlineStr">
+        <is>
+          <t>2026-03-22 01:28</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
✅ Veri Güncellendi:  - Mon Mar 23 01:28:44 UTC 2026
</commit_message>
<xml_diff>
--- a/leads_output.xlsx
+++ b/leads_output.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E359"/>
+  <dimension ref="A1:E362"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -10829,6 +10829,93 @@
         </is>
       </c>
     </row>
+    <row r="360">
+      <c r="A360" t="inlineStr">
+        <is>
+          <t>Eczane Esin</t>
+        </is>
+      </c>
+      <c r="B360" t="inlineStr">
+        <is>
+          <t>
++90 216 411 10 71</t>
+        </is>
+      </c>
+      <c r="C360" t="inlineStr">
+        <is>
+          <t>
+Sahrayı Cedit, Bahçeli Sk. No:5/A, 34734 Kadıköy/İstanbul, Türkiye</t>
+        </is>
+      </c>
+      <c r="D360" t="inlineStr">
+        <is>
+          <t>Kadikoy/Istanbul</t>
+        </is>
+      </c>
+      <c r="E360" t="inlineStr">
+        <is>
+          <t>2026-03-23 01:28</t>
+        </is>
+      </c>
+    </row>
+    <row r="361">
+      <c r="A361" t="inlineStr">
+        <is>
+          <t>Nilgün Eczanesi</t>
+        </is>
+      </c>
+      <c r="B361" t="inlineStr">
+        <is>
+          <t>
++90 216 467 80 50</t>
+        </is>
+      </c>
+      <c r="C361" t="inlineStr">
+        <is>
+          <t>
+Caddebostan, Bağdat Cad. No:1 D:B, 34728 Kadıköy/İstanbul, Türkiye</t>
+        </is>
+      </c>
+      <c r="D361" t="inlineStr">
+        <is>
+          <t>Kadikoy/Istanbul</t>
+        </is>
+      </c>
+      <c r="E361" t="inlineStr">
+        <is>
+          <t>2026-03-23 01:28</t>
+        </is>
+      </c>
+    </row>
+    <row r="362">
+      <c r="A362" t="inlineStr">
+        <is>
+          <t>Bal Eczanesi</t>
+        </is>
+      </c>
+      <c r="B362" t="inlineStr">
+        <is>
+          <t>
++90 216 766 44 51</t>
+        </is>
+      </c>
+      <c r="C362" t="inlineStr">
+        <is>
+          <t>
+Merdivenköy, Hızırbey Cd. No:160/D, 34732 Kadıköy/İstanbul, Türkiye</t>
+        </is>
+      </c>
+      <c r="D362" t="inlineStr">
+        <is>
+          <t>Kadikoy/Istanbul</t>
+        </is>
+      </c>
+      <c r="E362" t="inlineStr">
+        <is>
+          <t>2026-03-23 01:28</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
✅ Veri Güncellendi:  - Tue Mar 24 01:22:53 UTC 2026
</commit_message>
<xml_diff>
--- a/leads_output.xlsx
+++ b/leads_output.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E362"/>
+  <dimension ref="A1:E363"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -10916,6 +10916,35 @@
         </is>
       </c>
     </row>
+    <row r="363">
+      <c r="A363" t="inlineStr">
+        <is>
+          <t>Sezgi Eczanesi</t>
+        </is>
+      </c>
+      <c r="B363" t="inlineStr">
+        <is>
+          <t>
++90 216 629 62 69</t>
+        </is>
+      </c>
+      <c r="C363" t="inlineStr">
+        <is>
+          <t>
+Suadiye, Çolak İsmail Sk. 26/A, 34740 Kadıköy/İstanbul, Türkiye</t>
+        </is>
+      </c>
+      <c r="D363" t="inlineStr">
+        <is>
+          <t>Kadikoy/Istanbul</t>
+        </is>
+      </c>
+      <c r="E363" t="inlineStr">
+        <is>
+          <t>2026-03-24 01:22</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
✅ Veri Güncellendi:  - Wed Mar 25 01:27:11 UTC 2026
</commit_message>
<xml_diff>
--- a/leads_output.xlsx
+++ b/leads_output.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E363"/>
+  <dimension ref="A1:E364"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -10945,6 +10945,35 @@
         </is>
       </c>
     </row>
+    <row r="364">
+      <c r="A364" t="inlineStr">
+        <is>
+          <t>Gizem Eczanesi</t>
+        </is>
+      </c>
+      <c r="B364" t="inlineStr">
+        <is>
+          <t>
++90 216 208 32 91</t>
+        </is>
+      </c>
+      <c r="C364" t="inlineStr">
+        <is>
+          <t>
+Erenköy, Erenköy İstasyon Cd. No:35/E, 34738 Kadıköy/İstanbul, Türkiye</t>
+        </is>
+      </c>
+      <c r="D364" t="inlineStr">
+        <is>
+          <t>Kadikoy/Istanbul</t>
+        </is>
+      </c>
+      <c r="E364" t="inlineStr">
+        <is>
+          <t>2026-03-25 01:27</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
✅ Veri Güncellendi:  - Thu Mar 26 01:46:26 UTC 2026
</commit_message>
<xml_diff>
--- a/leads_output.xlsx
+++ b/leads_output.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E364"/>
+  <dimension ref="A1:E365"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -10974,6 +10974,35 @@
         </is>
       </c>
     </row>
+    <row r="365">
+      <c r="A365" t="inlineStr">
+        <is>
+          <t>Öze Dönüş Eczanesi</t>
+        </is>
+      </c>
+      <c r="B365" t="inlineStr">
+        <is>
+          <t>
++90 541 340 66 42</t>
+        </is>
+      </c>
+      <c r="C365" t="inlineStr">
+        <is>
+          <t>
+Acıbadem, Ata Sk. 10A, 34718 Kadıköy/İstanbul, Türkiye</t>
+        </is>
+      </c>
+      <c r="D365" t="inlineStr">
+        <is>
+          <t>Kadikoy/Istanbul</t>
+        </is>
+      </c>
+      <c r="E365" t="inlineStr">
+        <is>
+          <t>2026-03-26 01:46</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
✅ Veri Güncellendi:  - Fri Mar 27 01:46:42 UTC 2026
</commit_message>
<xml_diff>
--- a/leads_output.xlsx
+++ b/leads_output.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E365"/>
+  <dimension ref="A1:E368"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -11003,6 +11003,93 @@
         </is>
       </c>
     </row>
+    <row r="366">
+      <c r="A366" t="inlineStr">
+        <is>
+          <t>Gülnaz Eczanesi</t>
+        </is>
+      </c>
+      <c r="B366" t="inlineStr">
+        <is>
+          <t>
++90 216 755 90 55</t>
+        </is>
+      </c>
+      <c r="C366" t="inlineStr">
+        <is>
+          <t>
+Kozyatağı, Kaya Sultan Sokağı No: 24/A, 34742 Kadıköy/İstanbul, Türkiye</t>
+        </is>
+      </c>
+      <c r="D366" t="inlineStr">
+        <is>
+          <t>Kadikoy/Istanbul</t>
+        </is>
+      </c>
+      <c r="E366" t="inlineStr">
+        <is>
+          <t>2026-03-27 01:46</t>
+        </is>
+      </c>
+    </row>
+    <row r="367">
+      <c r="A367" t="inlineStr">
+        <is>
+          <t>CADDE GAMZE ECZANESİ-Ecz.Gamze Odabaşı Kılıçkaya</t>
+        </is>
+      </c>
+      <c r="B367" t="inlineStr">
+        <is>
+          <t>
++90 216 755 30 01</t>
+        </is>
+      </c>
+      <c r="C367" t="inlineStr">
+        <is>
+          <t>
+Caddebostan, Bağdat Cad. No:250, 34728 Kadıköy/İstanbul, Türkiye</t>
+        </is>
+      </c>
+      <c r="D367" t="inlineStr">
+        <is>
+          <t>Kadikoy/Istanbul</t>
+        </is>
+      </c>
+      <c r="E367" t="inlineStr">
+        <is>
+          <t>2026-03-27 01:46</t>
+        </is>
+      </c>
+    </row>
+    <row r="368">
+      <c r="A368" t="inlineStr">
+        <is>
+          <t>Eczane Aşık</t>
+        </is>
+      </c>
+      <c r="B368" t="inlineStr">
+        <is>
+          <t>
++90 216 325 17 79</t>
+        </is>
+      </c>
+      <c r="C368" t="inlineStr">
+        <is>
+          <t>
+Koşuyolu Mh. No:10 Pk:34718 Kadıköy/istanbul, Kalfa Çeşmesi Sk., 34718 Kadıköy/İstanbul, Türkiye</t>
+        </is>
+      </c>
+      <c r="D368" t="inlineStr">
+        <is>
+          <t>Kadikoy/Istanbul</t>
+        </is>
+      </c>
+      <c r="E368" t="inlineStr">
+        <is>
+          <t>2026-03-27 01:46</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
✅ Veri Güncellendi:  - Mon Mar 30 01:52:12 UTC 2026
</commit_message>
<xml_diff>
--- a/leads_output.xlsx
+++ b/leads_output.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E368"/>
+  <dimension ref="A1:E369"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -11090,6 +11090,35 @@
         </is>
       </c>
     </row>
+    <row r="369">
+      <c r="A369" t="inlineStr">
+        <is>
+          <t>Efes Eczanesi</t>
+        </is>
+      </c>
+      <c r="B369" t="inlineStr">
+        <is>
+          <t>
++90 216 362 57 16</t>
+        </is>
+      </c>
+      <c r="C369" t="inlineStr">
+        <is>
+          <t>
+Bostancı, Vukela Cd. No:30, 34744 Kadıköy/İstanbul - Asya, Türkiye</t>
+        </is>
+      </c>
+      <c r="D369" t="inlineStr">
+        <is>
+          <t>Kadikoy/Istanbul</t>
+        </is>
+      </c>
+      <c r="E369" t="inlineStr">
+        <is>
+          <t>2026-03-30 01:52</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
✅ Veri Güncellendi:  - Tue Mar 31 01:47:43 UTC 2026
</commit_message>
<xml_diff>
--- a/leads_output.xlsx
+++ b/leads_output.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E369"/>
+  <dimension ref="A1:E370"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -11119,6 +11119,35 @@
         </is>
       </c>
     </row>
+    <row r="370">
+      <c r="A370" t="inlineStr">
+        <is>
+          <t>ATA ECZANESİ - ATA PHARMACY - ATA APOTHEKE</t>
+        </is>
+      </c>
+      <c r="B370" t="inlineStr">
+        <is>
+          <t>
++90 216 567 57 60</t>
+        </is>
+      </c>
+      <c r="C370" t="inlineStr">
+        <is>
+          <t>
+Merdivenköy, Fahrettin Kerim Gökay Cd No:219/A, 34732 Kadıköy/İstanbul, Türkiye</t>
+        </is>
+      </c>
+      <c r="D370" t="inlineStr">
+        <is>
+          <t>Kadikoy/Istanbul</t>
+        </is>
+      </c>
+      <c r="E370" t="inlineStr">
+        <is>
+          <t>2026-03-31 01:47</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
✅ Veri Güncellendi:  - Wed Apr  1 01:55:07 UTC 2026
</commit_message>
<xml_diff>
--- a/leads_output.xlsx
+++ b/leads_output.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E370"/>
+  <dimension ref="A1:E372"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -11148,6 +11148,64 @@
         </is>
       </c>
     </row>
+    <row r="371">
+      <c r="A371" t="inlineStr">
+        <is>
+          <t>Berül Eczanesi</t>
+        </is>
+      </c>
+      <c r="B371" t="inlineStr">
+        <is>
+          <t>
++90 216 356 18 19</t>
+        </is>
+      </c>
+      <c r="C371" t="inlineStr">
+        <is>
+          <t>
+Suadiye, Çolak İsmail Sk. NO:15G, 34740 Kadıköy/İstanbul, Türkiye</t>
+        </is>
+      </c>
+      <c r="D371" t="inlineStr">
+        <is>
+          <t>Kadikoy/Istanbul</t>
+        </is>
+      </c>
+      <c r="E371" t="inlineStr">
+        <is>
+          <t>2026-04-01 01:55</t>
+        </is>
+      </c>
+    </row>
+    <row r="372">
+      <c r="A372" t="inlineStr">
+        <is>
+          <t>Fazlıoğlu Eczanesi</t>
+        </is>
+      </c>
+      <c r="B372" t="inlineStr">
+        <is>
+          <t>
++90 216 336 03 56</t>
+        </is>
+      </c>
+      <c r="C372" t="inlineStr">
+        <is>
+          <t>
+Acıbadem, Şemi Bey Sk. 2/c, 34718 Kadıköy/İstanbul, Türkiye</t>
+        </is>
+      </c>
+      <c r="D372" t="inlineStr">
+        <is>
+          <t>Kadikoy/Istanbul</t>
+        </is>
+      </c>
+      <c r="E372" t="inlineStr">
+        <is>
+          <t>2026-04-01 01:55</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
✅ Veri Güncellendi:  - Thu Apr  2 01:31:10 UTC 2026
</commit_message>
<xml_diff>
--- a/leads_output.xlsx
+++ b/leads_output.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E372"/>
+  <dimension ref="A1:E373"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -11206,6 +11206,35 @@
         </is>
       </c>
     </row>
+    <row r="373">
+      <c r="A373" t="inlineStr">
+        <is>
+          <t>Eczane Uzun Bostancı</t>
+        </is>
+      </c>
+      <c r="B373" t="inlineStr">
+        <is>
+          <t>
++90 216 372 80 01</t>
+        </is>
+      </c>
+      <c r="C373" t="inlineStr">
+        <is>
+          <t>
+Bostancı, Bağdat Cad. No: 538A, 34744 Kadıköy/İstanbul, Türkiye</t>
+        </is>
+      </c>
+      <c r="D373" t="inlineStr">
+        <is>
+          <t>Kadikoy/Istanbul</t>
+        </is>
+      </c>
+      <c r="E373" t="inlineStr">
+        <is>
+          <t>2026-04-02 01:31</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
✅ Veri Güncellendi:  - Sat Apr  4 01:27:28 UTC 2026
</commit_message>
<xml_diff>
--- a/leads_output.xlsx
+++ b/leads_output.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E373"/>
+  <dimension ref="A1:E375"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -11235,6 +11235,64 @@
         </is>
       </c>
     </row>
+    <row r="374">
+      <c r="A374" t="inlineStr">
+        <is>
+          <t>Mahur Eczanesi</t>
+        </is>
+      </c>
+      <c r="B374" t="inlineStr">
+        <is>
+          <t>
++90 216 771 27 85</t>
+        </is>
+      </c>
+      <c r="C374" t="inlineStr">
+        <is>
+          <t>
+Fenerbahçe mah. Bağdat cad, Mahur Sk. No:15/B, 34726 Kadıköy, Türkiye</t>
+        </is>
+      </c>
+      <c r="D374" t="inlineStr">
+        <is>
+          <t>Kadikoy/Istanbul</t>
+        </is>
+      </c>
+      <c r="E374" t="inlineStr">
+        <is>
+          <t>2026-04-04 01:27</t>
+        </is>
+      </c>
+    </row>
+    <row r="375">
+      <c r="A375" t="inlineStr">
+        <is>
+          <t>Haşanpaşa Eczanesi</t>
+        </is>
+      </c>
+      <c r="B375" t="inlineStr">
+        <is>
+          <t>
++90 216 370 75 25</t>
+        </is>
+      </c>
+      <c r="C375" t="inlineStr">
+        <is>
+          <t>
+Hasanpaşa, Kurbağalıdere Cd. 68/B, 34722 Kadıköy/İstanbul, Türkiye</t>
+        </is>
+      </c>
+      <c r="D375" t="inlineStr">
+        <is>
+          <t>Kadikoy/Istanbul</t>
+        </is>
+      </c>
+      <c r="E375" t="inlineStr">
+        <is>
+          <t>2026-04-04 01:27</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
✅ Veri Güncellendi:  - Wed Apr  8 01:48:55 UTC 2026
</commit_message>
<xml_diff>
--- a/leads_output.xlsx
+++ b/leads_output.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E375"/>
+  <dimension ref="A1:E376"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -11293,6 +11293,35 @@
         </is>
       </c>
     </row>
+    <row r="376">
+      <c r="A376" t="inlineStr">
+        <is>
+          <t>Rüya Eczanesi</t>
+        </is>
+      </c>
+      <c r="B376" t="inlineStr">
+        <is>
+          <t>
++90 216 658 61 80</t>
+        </is>
+      </c>
+      <c r="C376" t="inlineStr">
+        <is>
+          <t>
+19 Mayıs, Okur Sk. No:11, 34736 Kadıköy/İstanbul, Türkiye</t>
+        </is>
+      </c>
+      <c r="D376" t="inlineStr">
+        <is>
+          <t>Kadikoy/Istanbul</t>
+        </is>
+      </c>
+      <c r="E376" t="inlineStr">
+        <is>
+          <t>2026-04-08 01:48</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
✅ Veri Güncellendi:  - Fri Apr 10 01:52:39 UTC 2026
</commit_message>
<xml_diff>
--- a/leads_output.xlsx
+++ b/leads_output.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E376"/>
+  <dimension ref="A1:E377"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -11322,6 +11322,35 @@
         </is>
       </c>
     </row>
+    <row r="377">
+      <c r="A377" t="inlineStr">
+        <is>
+          <t>Yeşilbahar Eczanesi</t>
+        </is>
+      </c>
+      <c r="B377" t="inlineStr">
+        <is>
+          <t>
++90 216 360 61 54</t>
+        </is>
+      </c>
+      <c r="C377" t="inlineStr">
+        <is>
+          <t>
+Kozyatağı, Korkut Sk. No:6\A, 34730 Kadıköy/İstanbul, Türkiye</t>
+        </is>
+      </c>
+      <c r="D377" t="inlineStr">
+        <is>
+          <t>Kadikoy/Istanbul</t>
+        </is>
+      </c>
+      <c r="E377" t="inlineStr">
+        <is>
+          <t>2026-04-10 01:52</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
✅ Veri Güncellendi:  - Sat Apr 11 01:30:40 UTC 2026
</commit_message>
<xml_diff>
--- a/leads_output.xlsx
+++ b/leads_output.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E377"/>
+  <dimension ref="A1:E378"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -11351,6 +11351,35 @@
         </is>
       </c>
     </row>
+    <row r="378">
+      <c r="A378" t="inlineStr">
+        <is>
+          <t>Nazlım eczanesi</t>
+        </is>
+      </c>
+      <c r="B378" t="inlineStr">
+        <is>
+          <t>
++90 216 478 00 30</t>
+        </is>
+      </c>
+      <c r="C378" t="inlineStr">
+        <is>
+          <t>
+Erenköy, Fırın Sk. no:30/A, 34738 Kadıköy/İstanbul, Türkiye</t>
+        </is>
+      </c>
+      <c r="D378" t="inlineStr">
+        <is>
+          <t>Kadikoy/Istanbul</t>
+        </is>
+      </c>
+      <c r="E378" t="inlineStr">
+        <is>
+          <t>2026-04-11 01:30</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
✅ Veri Güncellendi:  - Mon Apr 13 02:00:10 UTC 2026
</commit_message>
<xml_diff>
--- a/leads_output.xlsx
+++ b/leads_output.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E378"/>
+  <dimension ref="A1:E380"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -11380,6 +11380,64 @@
         </is>
       </c>
     </row>
+    <row r="379">
+      <c r="A379" t="inlineStr">
+        <is>
+          <t>Erenköy Eczanesi</t>
+        </is>
+      </c>
+      <c r="B379" t="inlineStr">
+        <is>
+          <t>
++90 505 029 62 29</t>
+        </is>
+      </c>
+      <c r="C379" t="inlineStr">
+        <is>
+          <t>
+Göztepe, Tütüncü Mehmet Efendi Cd. No:78 D:B, 34730 Kadıköy/İstanbul, Türkiye</t>
+        </is>
+      </c>
+      <c r="D379" t="inlineStr">
+        <is>
+          <t>Kadikoy/Istanbul</t>
+        </is>
+      </c>
+      <c r="E379" t="inlineStr">
+        <is>
+          <t>2026-04-13 02:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="380">
+      <c r="A380" t="inlineStr">
+        <is>
+          <t>Doğa Eczanesi</t>
+        </is>
+      </c>
+      <c r="B380" t="inlineStr">
+        <is>
+          <t>
++90 216 338 44 38</t>
+        </is>
+      </c>
+      <c r="C380" t="inlineStr">
+        <is>
+          <t>
+Fenerbahçe, Fener Kalamış Cd. NO:2-4/B, 34726 Kadıköy/İstanbul, Türkiye</t>
+        </is>
+      </c>
+      <c r="D380" t="inlineStr">
+        <is>
+          <t>Kadikoy/Istanbul</t>
+        </is>
+      </c>
+      <c r="E380" t="inlineStr">
+        <is>
+          <t>2026-04-13 02:00</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
✅ Veri Güncellendi:  - Sun Apr 19 01:59:07 UTC 2026
</commit_message>
<xml_diff>
--- a/leads_output.xlsx
+++ b/leads_output.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E380"/>
+  <dimension ref="A1:E381"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -11438,6 +11438,35 @@
         </is>
       </c>
     </row>
+    <row r="381">
+      <c r="A381" t="inlineStr">
+        <is>
+          <t>Tuğçe Eczanesi</t>
+        </is>
+      </c>
+      <c r="B381" t="inlineStr">
+        <is>
+          <t>
++90 216 363 87 85</t>
+        </is>
+      </c>
+      <c r="C381" t="inlineStr">
+        <is>
+          <t>
+Fenerbahçe Mahallesi Hasan Ali Yücel Sokak, Bağdat Cad. 15/A, 34726 Kadıköy/İstanbul, Türkiye</t>
+        </is>
+      </c>
+      <c r="D381" t="inlineStr">
+        <is>
+          <t>Kadikoy/Istanbul</t>
+        </is>
+      </c>
+      <c r="E381" t="inlineStr">
+        <is>
+          <t>2026-04-19 01:59</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
✅ Veri Güncellendi:  - Mon Apr 20 02:00:26 UTC 2026
</commit_message>
<xml_diff>
--- a/leads_output.xlsx
+++ b/leads_output.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E381"/>
+  <dimension ref="A1:E382"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -11467,6 +11467,35 @@
         </is>
       </c>
     </row>
+    <row r="382">
+      <c r="A382" t="inlineStr">
+        <is>
+          <t>Şeker Eczanesi</t>
+        </is>
+      </c>
+      <c r="B382" t="inlineStr">
+        <is>
+          <t>
++90 216 369 81 98</t>
+        </is>
+      </c>
+      <c r="C382" t="inlineStr">
+        <is>
+          <t>
+Göztepe, Fahrettin Kerim Gökay Cd No:260, 34730 Kadıköy/İstanbul, Türkiye</t>
+        </is>
+      </c>
+      <c r="D382" t="inlineStr">
+        <is>
+          <t>Kadikoy/Istanbul</t>
+        </is>
+      </c>
+      <c r="E382" t="inlineStr">
+        <is>
+          <t>2026-04-20 02:00</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
✅ Veri Güncellendi:  - Fri May  1 02:25:57 UTC 2026
</commit_message>
<xml_diff>
--- a/leads_output.xlsx
+++ b/leads_output.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E382"/>
+  <dimension ref="A1:E383"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -11496,6 +11496,35 @@
         </is>
       </c>
     </row>
+    <row r="383">
+      <c r="A383" t="inlineStr">
+        <is>
+          <t>Deniz Eczanesi</t>
+        </is>
+      </c>
+      <c r="B383" t="inlineStr">
+        <is>
+          <t>
++90 216 348 11 28</t>
+        </is>
+      </c>
+      <c r="C383" t="inlineStr">
+        <is>
+          <t>
+Feneryolu, Bağdat Cad. 73/B, 34724 Kadıköy/İstanbul, Türkiye</t>
+        </is>
+      </c>
+      <c r="D383" t="inlineStr">
+        <is>
+          <t>Kadikoy/Istanbul</t>
+        </is>
+      </c>
+      <c r="E383" t="inlineStr">
+        <is>
+          <t>2026-05-01 02:25</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
✅ Veri Güncellendi:  - Sun May 10 02:12:00 UTC 2026
</commit_message>
<xml_diff>
--- a/leads_output.xlsx
+++ b/leads_output.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E383"/>
+  <dimension ref="A1:E384"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -11525,6 +11525,35 @@
         </is>
       </c>
     </row>
+    <row r="384">
+      <c r="A384" t="inlineStr">
+        <is>
+          <t>Marmara eczanesi</t>
+        </is>
+      </c>
+      <c r="B384" t="inlineStr">
+        <is>
+          <t>
++90 216 567 70 30</t>
+        </is>
+      </c>
+      <c r="C384" t="inlineStr">
+        <is>
+          <t>
+Feneryolu, Fahrettin Kerim Gökay Cd 146/A, 34732 Kadıköy/İstanbul, Türkiye</t>
+        </is>
+      </c>
+      <c r="D384" t="inlineStr">
+        <is>
+          <t>Kadikoy/Istanbul</t>
+        </is>
+      </c>
+      <c r="E384" t="inlineStr">
+        <is>
+          <t>2026-05-10 02:11</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
✅ Veri Güncellendi:  - Mon May 11 02:30:25 UTC 2026
</commit_message>
<xml_diff>
--- a/leads_output.xlsx
+++ b/leads_output.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E384"/>
+  <dimension ref="A1:E385"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -11554,6 +11554,35 @@
         </is>
       </c>
     </row>
+    <row r="385">
+      <c r="A385" t="inlineStr">
+        <is>
+          <t>İncir Eczanesi</t>
+        </is>
+      </c>
+      <c r="B385" t="inlineStr">
+        <is>
+          <t>
++90 549 546 24 70</t>
+        </is>
+      </c>
+      <c r="C385" t="inlineStr">
+        <is>
+          <t>
+19 Mayıs, Yazar Sokağı 7/B, 34736 Kadıköy/İstanbul, Türkiye</t>
+        </is>
+      </c>
+      <c r="D385" t="inlineStr">
+        <is>
+          <t>Kadikoy/Istanbul</t>
+        </is>
+      </c>
+      <c r="E385" t="inlineStr">
+        <is>
+          <t>2026-05-11 02:30</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
✅ Veri Güncellendi:  - Tue May 12 02:15:41 UTC 2026
</commit_message>
<xml_diff>
--- a/leads_output.xlsx
+++ b/leads_output.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E385"/>
+  <dimension ref="A1:E386"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -11583,6 +11583,35 @@
         </is>
       </c>
     </row>
+    <row r="386">
+      <c r="A386" t="inlineStr">
+        <is>
+          <t>MAYA ECZANESİ</t>
+        </is>
+      </c>
+      <c r="B386" t="inlineStr">
+        <is>
+          <t>
++90 546 416 62 92</t>
+        </is>
+      </c>
+      <c r="C386" t="inlineStr">
+        <is>
+          <t>
+Bostancı, Bağdat Cad. NO:478/C, 34000 Kadıköy/İstanbul, Türkiye</t>
+        </is>
+      </c>
+      <c r="D386" t="inlineStr">
+        <is>
+          <t>Kadikoy/Istanbul</t>
+        </is>
+      </c>
+      <c r="E386" t="inlineStr">
+        <is>
+          <t>2026-05-12 02:15</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
✅ Veri Güncellendi:  - Fri May 15 02:31:01 UTC 2026
</commit_message>
<xml_diff>
--- a/leads_output.xlsx
+++ b/leads_output.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E386"/>
+  <dimension ref="A1:E387"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -11612,6 +11612,35 @@
         </is>
       </c>
     </row>
+    <row r="387">
+      <c r="A387" t="inlineStr">
+        <is>
+          <t>Eczane Suadiye Çağla</t>
+        </is>
+      </c>
+      <c r="B387" t="inlineStr">
+        <is>
+          <t>
++90 216 362 55 09</t>
+        </is>
+      </c>
+      <c r="C387" t="inlineStr">
+        <is>
+          <t>
+Suadiye, Emin Ali Paşa Cd. No:44 D:B, 34740 Kadıköy/İstanbul, Türkiye</t>
+        </is>
+      </c>
+      <c r="D387" t="inlineStr">
+        <is>
+          <t>Kadikoy/Istanbul</t>
+        </is>
+      </c>
+      <c r="E387" t="inlineStr">
+        <is>
+          <t>2026-05-15 02:31</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
✅ Veri Güncellendi:  - Sat May 16 02:13:04 UTC 2026
</commit_message>
<xml_diff>
--- a/leads_output.xlsx
+++ b/leads_output.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E387"/>
+  <dimension ref="A1:E388"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -11641,6 +11641,35 @@
         </is>
       </c>
     </row>
+    <row r="388">
+      <c r="A388" t="inlineStr">
+        <is>
+          <t>Kristal Eczanesi</t>
+        </is>
+      </c>
+      <c r="B388" t="inlineStr">
+        <is>
+          <t>
++90 216 362 41 64</t>
+        </is>
+      </c>
+      <c r="C388" t="inlineStr">
+        <is>
+          <t>
+Kozyatağı Mh.Kocayol Caddesi, Kozyatağı, Seda Sk. No:8, 34742 Kadıköy/İstanbul, Türkiye</t>
+        </is>
+      </c>
+      <c r="D388" t="inlineStr">
+        <is>
+          <t>Kadikoy/Istanbul</t>
+        </is>
+      </c>
+      <c r="E388" t="inlineStr">
+        <is>
+          <t>2026-05-16 02:13</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
✅ Veri Güncellendi:  - Tue May 19 02:37:00 UTC 2026
</commit_message>
<xml_diff>
--- a/leads_output.xlsx
+++ b/leads_output.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E388"/>
+  <dimension ref="A1:E390"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -11670,6 +11670,64 @@
         </is>
       </c>
     </row>
+    <row r="389">
+      <c r="A389" t="inlineStr">
+        <is>
+          <t>Zeynep Eczanesi</t>
+        </is>
+      </c>
+      <c r="B389" t="inlineStr">
+        <is>
+          <t>
++90 532 429 47 45</t>
+        </is>
+      </c>
+      <c r="C389" t="inlineStr">
+        <is>
+          <t>
+Merdivenköy, Günaydın Sokağı No:7/C, 34732 Kadıköy/İstanbul, Türkiye</t>
+        </is>
+      </c>
+      <c r="D389" t="inlineStr">
+        <is>
+          <t>Kadikoy/Istanbul</t>
+        </is>
+      </c>
+      <c r="E389" t="inlineStr">
+        <is>
+          <t>2026-05-19 02:36</t>
+        </is>
+      </c>
+    </row>
+    <row r="390">
+      <c r="A390" t="inlineStr">
+        <is>
+          <t>Eczane Serdil</t>
+        </is>
+      </c>
+      <c r="B390" t="inlineStr">
+        <is>
+          <t>
++90 216 565 80 01</t>
+        </is>
+      </c>
+      <c r="C390" t="inlineStr">
+        <is>
+          <t>
+Feneryolu, Fahrettin Kerim Gökay Cd No:142/B, 34724 Kadıköy/İstanbul, Türkiye</t>
+        </is>
+      </c>
+      <c r="D390" t="inlineStr">
+        <is>
+          <t>Kadikoy/Istanbul</t>
+        </is>
+      </c>
+      <c r="E390" t="inlineStr">
+        <is>
+          <t>2026-05-19 02:37</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
✅ Veri Güncellendi:  - Wed May 20 02:37:07 UTC 2026
</commit_message>
<xml_diff>
--- a/leads_output.xlsx
+++ b/leads_output.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E390"/>
+  <dimension ref="A1:E391"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -11728,6 +11728,35 @@
         </is>
       </c>
     </row>
+    <row r="391">
+      <c r="A391" t="inlineStr">
+        <is>
+          <t>Sefa Eczanesi</t>
+        </is>
+      </c>
+      <c r="B391" t="inlineStr">
+        <is>
+          <t>
++90 216 567 01 08</t>
+        </is>
+      </c>
+      <c r="C391" t="inlineStr">
+        <is>
+          <t>
+Dumlupınar mah Hızırbey Caddes. No:203-205/B-C, Kadıköy/İstanbul, Türkiye</t>
+        </is>
+      </c>
+      <c r="D391" t="inlineStr">
+        <is>
+          <t>Kadikoy/Istanbul</t>
+        </is>
+      </c>
+      <c r="E391" t="inlineStr">
+        <is>
+          <t>2026-05-20 02:37</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
✅ Veri Güncellendi:  - Sat May 30 02:28:43 UTC 2026
</commit_message>
<xml_diff>
--- a/leads_output.xlsx
+++ b/leads_output.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E391"/>
+  <dimension ref="A1:E392"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -11757,6 +11757,35 @@
         </is>
       </c>
     </row>
+    <row r="392">
+      <c r="A392" t="inlineStr">
+        <is>
+          <t>BAĞDAT YAŞAM ECZANESİ</t>
+        </is>
+      </c>
+      <c r="B392" t="inlineStr">
+        <is>
+          <t>
++90 539 273 15 24</t>
+        </is>
+      </c>
+      <c r="C392" t="inlineStr">
+        <is>
+          <t>
+Fenerbahçe, Dr. Faruk Ayanoğlu Cd. No:2 D:A, 34726 Kadıköy/İstanbul, Türkiye</t>
+        </is>
+      </c>
+      <c r="D392" t="inlineStr">
+        <is>
+          <t>Kadikoy/Istanbul</t>
+        </is>
+      </c>
+      <c r="E392" t="inlineStr">
+        <is>
+          <t>2026-05-30 02:28</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
✅ Veri Güncellendi:  - Mon Jun  1 02:54:20 UTC 2026
</commit_message>
<xml_diff>
--- a/leads_output.xlsx
+++ b/leads_output.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E392"/>
+  <dimension ref="A1:E394"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -11786,6 +11786,64 @@
         </is>
       </c>
     </row>
+    <row r="393">
+      <c r="A393" t="inlineStr">
+        <is>
+          <t>Ezgi Eczanesi</t>
+        </is>
+      </c>
+      <c r="B393" t="inlineStr">
+        <is>
+          <t>
++90 216 340 67 05</t>
+        </is>
+      </c>
+      <c r="C393" t="inlineStr">
+        <is>
+          <t>
+Fikirtepe, Mandıra Cd. No:60 D:C, 34720 Kadıköy/İstanbul, Türkiye</t>
+        </is>
+      </c>
+      <c r="D393" t="inlineStr">
+        <is>
+          <t>Kadikoy/Istanbul</t>
+        </is>
+      </c>
+      <c r="E393" t="inlineStr">
+        <is>
+          <t>2026-06-01 02:54</t>
+        </is>
+      </c>
+    </row>
+    <row r="394">
+      <c r="A394" t="inlineStr">
+        <is>
+          <t>Bostancı Cadde Eczanesi ( English Speaking Pharmacy) APOTHEKE</t>
+        </is>
+      </c>
+      <c r="B394" t="inlineStr">
+        <is>
+          <t>
++90 532 522 25 35</t>
+        </is>
+      </c>
+      <c r="C394" t="inlineStr">
+        <is>
+          <t>
+Bostancı, Prof. Dr. Ali Nihat Tarlan Cd No:43D, 34744 Kadıköy/İstanbul, Türkiye</t>
+        </is>
+      </c>
+      <c r="D394" t="inlineStr">
+        <is>
+          <t>Kadikoy/Istanbul</t>
+        </is>
+      </c>
+      <c r="E394" t="inlineStr">
+        <is>
+          <t>2026-06-01 02:54</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
✅ Veri Güncellendi:  - Tue Jun  2 02:51:18 UTC 2026
</commit_message>
<xml_diff>
--- a/leads_output.xlsx
+++ b/leads_output.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E394"/>
+  <dimension ref="A1:E395"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -11844,6 +11844,35 @@
         </is>
       </c>
     </row>
+    <row r="395">
+      <c r="A395" t="inlineStr">
+        <is>
+          <t>SEZGİNER ECZANESİ (English Spoken Pharmacy)</t>
+        </is>
+      </c>
+      <c r="B395" t="inlineStr">
+        <is>
+          <t>
++90 501 943 84 31</t>
+        </is>
+      </c>
+      <c r="C395" t="inlineStr">
+        <is>
+          <t>
+Sahrayı Cedit, Halk Sk. No:14, 34734 Kadıköy/İstanbul, Türkiye</t>
+        </is>
+      </c>
+      <c r="D395" t="inlineStr">
+        <is>
+          <t>Kadikoy/Istanbul</t>
+        </is>
+      </c>
+      <c r="E395" t="inlineStr">
+        <is>
+          <t>2026-06-02 02:51</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
✅ Veri Güncellendi:  - Wed Jun 10 02:43:14 UTC 2026
</commit_message>
<xml_diff>
--- a/leads_output.xlsx
+++ b/leads_output.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E395"/>
+  <dimension ref="A1:E396"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -11873,6 +11873,35 @@
         </is>
       </c>
     </row>
+    <row r="396">
+      <c r="A396" t="inlineStr">
+        <is>
+          <t>Bilgen Eczanesi</t>
+        </is>
+      </c>
+      <c r="B396" t="inlineStr">
+        <is>
+          <t>
++90 532 368 47 45</t>
+        </is>
+      </c>
+      <c r="C396" t="inlineStr">
+        <is>
+          <t>
+SAHRAYICEDİT MAH. ATATÜRK CAD, ATATÜRK CADDESİ ÜZERİNDE VESTEL VE DİŞ POLİKLİNİĞİ OLAN 7 NOLU OPTİMUM APARTMANINI GEÇTİKTEN HEMEN SONRAKİ SOKAĞIN BAŞI -APARTMANIN YAN TARAFINDA KALAN DÜKKANIDIR, Taşlıyol Sk. NO:2 D:1A, 34734 Kadıköy/İstanbul, Türkiye</t>
+        </is>
+      </c>
+      <c r="D396" t="inlineStr">
+        <is>
+          <t>Kadikoy/Istanbul</t>
+        </is>
+      </c>
+      <c r="E396" t="inlineStr">
+        <is>
+          <t>2026-06-10 02:43</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
✅ Veri Güncellendi:  - Wed Jun 17 02:56:01 UTC 2026
</commit_message>
<xml_diff>
--- a/leads_output.xlsx
+++ b/leads_output.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E396"/>
+  <dimension ref="A1:E397"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -11902,6 +11902,35 @@
         </is>
       </c>
     </row>
+    <row r="397">
+      <c r="A397" t="inlineStr">
+        <is>
+          <t>Özdemir Eczanesi</t>
+        </is>
+      </c>
+      <c r="B397" t="inlineStr">
+        <is>
+          <t>
++90 546 642 15 05</t>
+        </is>
+      </c>
+      <c r="C397" t="inlineStr">
+        <is>
+          <t>
+optimist residence özdemir eczanesi, Fikirtepe, Rüzgar Sk. No:10/46, 34720 Kadıköy/İstanbul, Türkiye</t>
+        </is>
+      </c>
+      <c r="D397" t="inlineStr">
+        <is>
+          <t>Kadikoy/Istanbul</t>
+        </is>
+      </c>
+      <c r="E397" t="inlineStr">
+        <is>
+          <t>2026-06-17 02:56</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
✅ Veri Güncellendi:  - Sat Jun 20 02:40:26 UTC 2026
</commit_message>
<xml_diff>
--- a/leads_output.xlsx
+++ b/leads_output.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E397"/>
+  <dimension ref="A1:E398"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -11931,6 +11931,35 @@
         </is>
       </c>
     </row>
+    <row r="398">
+      <c r="A398" t="inlineStr">
+        <is>
+          <t>Eczane Ertürk</t>
+        </is>
+      </c>
+      <c r="B398" t="inlineStr">
+        <is>
+          <t>
++90 216 363 61 39</t>
+        </is>
+      </c>
+      <c r="C398" t="inlineStr">
+        <is>
+          <t>
+Erenköy, Ethemefendi Cad. no: 78/A, 34738 Kadıköy/İstanbul, Türkiye</t>
+        </is>
+      </c>
+      <c r="D398" t="inlineStr">
+        <is>
+          <t>Kadikoy/Istanbul</t>
+        </is>
+      </c>
+      <c r="E398" t="inlineStr">
+        <is>
+          <t>2026-06-20 02:40</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
✅ Veri Güncellendi:  - Fri Jun 26 02:39:31 UTC 2026
</commit_message>
<xml_diff>
--- a/leads_output.xlsx
+++ b/leads_output.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E398"/>
+  <dimension ref="A1:E399"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -11960,6 +11960,35 @@
         </is>
       </c>
     </row>
+    <row r="399">
+      <c r="A399" t="inlineStr">
+        <is>
+          <t>Organik Eczanesi</t>
+        </is>
+      </c>
+      <c r="B399" t="inlineStr">
+        <is>
+          <t>
++90 216 755 60 55</t>
+        </is>
+      </c>
+      <c r="C399" t="inlineStr">
+        <is>
+          <t>
+Feneryolu, Fahrettin Kerim Gökay Cd No:84/A, 34724 Kadıköy/İstanbul, Türkiye</t>
+        </is>
+      </c>
+      <c r="D399" t="inlineStr">
+        <is>
+          <t>Kadikoy/Istanbul</t>
+        </is>
+      </c>
+      <c r="E399" t="inlineStr">
+        <is>
+          <t>2026-06-26 02:39</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
✅ Veri Güncellendi:  - Mon Jul 13 02:01:53 UTC 2026
</commit_message>
<xml_diff>
--- a/leads_output.xlsx
+++ b/leads_output.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E399"/>
+  <dimension ref="A1:E400"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -11989,6 +11989,35 @@
         </is>
       </c>
     </row>
+    <row r="400">
+      <c r="A400" t="inlineStr">
+        <is>
+          <t>Sahra Eczanesi</t>
+        </is>
+      </c>
+      <c r="B400" t="inlineStr">
+        <is>
+          <t>
++90 216 360 34 44</t>
+        </is>
+      </c>
+      <c r="C400" t="inlineStr">
+        <is>
+          <t>
+Sahrayı Cedit, Halk Sk. No:46, 34734 Kadıköy/İstanbul, Türkiye</t>
+        </is>
+      </c>
+      <c r="D400" t="inlineStr">
+        <is>
+          <t>Kadikoy/Istanbul</t>
+        </is>
+      </c>
+      <c r="E400" t="inlineStr">
+        <is>
+          <t>2026-07-13 02:01</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
✅ Veri Güncellendi:  - Tue Jul 14 01:48:40 UTC 2026
</commit_message>
<xml_diff>
--- a/leads_output.xlsx
+++ b/leads_output.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E400"/>
+  <dimension ref="A1:E402"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -12018,6 +12018,64 @@
         </is>
       </c>
     </row>
+    <row r="401">
+      <c r="A401" t="inlineStr">
+        <is>
+          <t>Ezgi İzel Eczanesi</t>
+        </is>
+      </c>
+      <c r="B401" t="inlineStr">
+        <is>
+          <t>
++90 533 724 06 74</t>
+        </is>
+      </c>
+      <c r="C401" t="inlineStr">
+        <is>
+          <t>
+Sahrayı Cedit, Ferit Bey Sk. no:6/c, 34744 Kadıköy/İstanbul, Türkiye</t>
+        </is>
+      </c>
+      <c r="D401" t="inlineStr">
+        <is>
+          <t>Kadikoy/Istanbul</t>
+        </is>
+      </c>
+      <c r="E401" t="inlineStr">
+        <is>
+          <t>2026-07-14 01:48</t>
+        </is>
+      </c>
+    </row>
+    <row r="402">
+      <c r="A402" t="inlineStr">
+        <is>
+          <t>Acil Nöbetçi Eczane Moto-Kurye 7/24 - Pharmacy Delivery - Suadiye Eczane kurye İstanbul</t>
+        </is>
+      </c>
+      <c r="B402" t="inlineStr">
+        <is>
+          <t>
++90 544 668 24 11</t>
+        </is>
+      </c>
+      <c r="C402" t="inlineStr">
+        <is>
+          <t>
+Sahrayı Cedit, Bayar Cd. 5/A, 34734 Kadıköy/İstanbul, Türkiye</t>
+        </is>
+      </c>
+      <c r="D402" t="inlineStr">
+        <is>
+          <t>Kadikoy/Istanbul</t>
+        </is>
+      </c>
+      <c r="E402" t="inlineStr">
+        <is>
+          <t>2026-07-14 01:48</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
✅ Veri Güncellendi:  - Thu Jul 16 01:54:49 UTC 2026
</commit_message>
<xml_diff>
--- a/leads_output.xlsx
+++ b/leads_output.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E402"/>
+  <dimension ref="A1:E403"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -12076,6 +12076,35 @@
         </is>
       </c>
     </row>
+    <row r="403">
+      <c r="A403" t="inlineStr">
+        <is>
+          <t>ECZANE DOĞRU</t>
+        </is>
+      </c>
+      <c r="B403" t="inlineStr">
+        <is>
+          <t>
++90 216 410 04 26</t>
+        </is>
+      </c>
+      <c r="C403" t="inlineStr">
+        <is>
+          <t>
+Kozyatağı, Kaymakam Kemal Sk. 2/A, 34742 Kadıköy/İstanbul, Türkiye</t>
+        </is>
+      </c>
+      <c r="D403" t="inlineStr">
+        <is>
+          <t>Kadikoy/Istanbul</t>
+        </is>
+      </c>
+      <c r="E403" t="inlineStr">
+        <is>
+          <t>2026-07-16 01:54</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
✅ Veri Güncellendi:  - Fri Jul 17 01:59:31 UTC 2026
</commit_message>
<xml_diff>
--- a/leads_output.xlsx
+++ b/leads_output.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E403"/>
+  <dimension ref="A1:E404"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -12105,6 +12105,35 @@
         </is>
       </c>
     </row>
+    <row r="404">
+      <c r="A404" t="inlineStr">
+        <is>
+          <t>Lilyum Eczanesi</t>
+        </is>
+      </c>
+      <c r="B404" t="inlineStr">
+        <is>
+          <t>
++90 216 766 49 05</t>
+        </is>
+      </c>
+      <c r="C404" t="inlineStr">
+        <is>
+          <t>
+Feneryolu, Bağdat Cad. No:92B, 34724 Kadıköy/İstanbul, Türkiye</t>
+        </is>
+      </c>
+      <c r="D404" t="inlineStr">
+        <is>
+          <t>Kadikoy/Istanbul</t>
+        </is>
+      </c>
+      <c r="E404" t="inlineStr">
+        <is>
+          <t>2026-07-17 01:59</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
✅ Veri Güncellendi:  - Sat Jul 18 01:48:20 UTC 2026
</commit_message>
<xml_diff>
--- a/leads_output.xlsx
+++ b/leads_output.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E404"/>
+  <dimension ref="A1:E405"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -12134,6 +12134,35 @@
         </is>
       </c>
     </row>
+    <row r="405">
+      <c r="A405" t="inlineStr">
+        <is>
+          <t>ORGANİK ECZANESİ</t>
+        </is>
+      </c>
+      <c r="B405" t="inlineStr">
+        <is>
+          <t>
++90 216 755 60 55</t>
+        </is>
+      </c>
+      <c r="C405" t="inlineStr">
+        <is>
+          <t>
+Feneryolu, Fahrettin Kerim Gökay Cd Sevgili Apt No:84/A, 34724 Kadıköy/İstanbul, Türkiye</t>
+        </is>
+      </c>
+      <c r="D405" t="inlineStr">
+        <is>
+          <t>Kadikoy/Istanbul</t>
+        </is>
+      </c>
+      <c r="E405" t="inlineStr">
+        <is>
+          <t>2026-07-18 01:48</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
✅ Veri Güncellendi:  - Tue Jul 28 01:51:12 UTC 2026
</commit_message>
<xml_diff>
--- a/leads_output.xlsx
+++ b/leads_output.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E405"/>
+  <dimension ref="A1:E406"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -12163,6 +12163,35 @@
         </is>
       </c>
     </row>
+    <row r="406">
+      <c r="A406" t="inlineStr">
+        <is>
+          <t>ÇAĞLAR ECZANESİ</t>
+        </is>
+      </c>
+      <c r="B406" t="inlineStr">
+        <is>
+          <t>
++90 216 463 48 00</t>
+        </is>
+      </c>
+      <c r="C406" t="inlineStr">
+        <is>
+          <t>
+19 Mayıs, Okur Sk. No:11/B, 34736 Kadıköy/İstanbul, Türkiye</t>
+        </is>
+      </c>
+      <c r="D406" t="inlineStr">
+        <is>
+          <t>Kadikoy/Istanbul</t>
+        </is>
+      </c>
+      <c r="E406" t="inlineStr">
+        <is>
+          <t>2026-07-28 01:51</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
✅ Veri Güncellendi:  - Tue Aug  4 01:50:07 UTC 2026
</commit_message>
<xml_diff>
--- a/leads_output.xlsx
+++ b/leads_output.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E406"/>
+  <dimension ref="A1:E407"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -12192,6 +12192,35 @@
         </is>
       </c>
     </row>
+    <row r="407">
+      <c r="A407" t="inlineStr">
+        <is>
+          <t>Acıbadem Plus Eczanesi</t>
+        </is>
+      </c>
+      <c r="B407" t="inlineStr">
+        <is>
+          <t>
++90 216 326 50 72</t>
+        </is>
+      </c>
+      <c r="C407" t="inlineStr">
+        <is>
+          <t>
+Acıbadem, Acıbadem Cd. 116/A, 34718 Kadıköy/İstanbul, Türkiye</t>
+        </is>
+      </c>
+      <c r="D407" t="inlineStr">
+        <is>
+          <t>Kadikoy/Istanbul</t>
+        </is>
+      </c>
+      <c r="E407" t="inlineStr">
+        <is>
+          <t>2026-08-04 01:50</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
✅ Veri Güncellendi:  - Thu Aug  6 01:52:05 UTC 2026
</commit_message>
<xml_diff>
--- a/leads_output.xlsx
+++ b/leads_output.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E407"/>
+  <dimension ref="A1:E408"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -12221,6 +12221,35 @@
         </is>
       </c>
     </row>
+    <row r="408">
+      <c r="A408" t="inlineStr">
+        <is>
+          <t>Fito Eczane</t>
+        </is>
+      </c>
+      <c r="B408" t="inlineStr">
+        <is>
+          <t>
++90 216 418 44 15</t>
+        </is>
+      </c>
+      <c r="C408" t="inlineStr">
+        <is>
+          <t>
+Hasanpaşa, Söğütlüçeşme Cad. söğütlü han D:178/A, 34722 Kadıköy/İstanbul, Türkiye</t>
+        </is>
+      </c>
+      <c r="D408" t="inlineStr">
+        <is>
+          <t>Kadikoy/Istanbul</t>
+        </is>
+      </c>
+      <c r="E408" t="inlineStr">
+        <is>
+          <t>2026-08-06 01:52</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
✅ Veri Güncellendi:  - Sun Aug  9 01:07:17 UTC 2026
</commit_message>
<xml_diff>
--- a/leads_output.xlsx
+++ b/leads_output.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E408"/>
+  <dimension ref="A1:E409"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -12250,6 +12250,35 @@
         </is>
       </c>
     </row>
+    <row r="409">
+      <c r="A409" t="inlineStr">
+        <is>
+          <t>Alp Koray Eczanesi</t>
+        </is>
+      </c>
+      <c r="B409" t="inlineStr">
+        <is>
+          <t>
++90 216 414 19 74</t>
+        </is>
+      </c>
+      <c r="C409" t="inlineStr">
+        <is>
+          <t>
+Eğitim, Nahitbey Sok., 34722 Kadıköy/İstanbul, Türkiye</t>
+        </is>
+      </c>
+      <c r="D409" t="inlineStr">
+        <is>
+          <t>Kadikoy/Istanbul</t>
+        </is>
+      </c>
+      <c r="E409" t="inlineStr">
+        <is>
+          <t>2026-08-09 01:07</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
✅ Veri Güncellendi:  - Wed Aug 12 01:15:19 UTC 2026
</commit_message>
<xml_diff>
--- a/leads_output.xlsx
+++ b/leads_output.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E409"/>
+  <dimension ref="A1:E410"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -12279,6 +12279,35 @@
         </is>
       </c>
     </row>
+    <row r="410">
+      <c r="A410" t="inlineStr">
+        <is>
+          <t>Seden Eczanesi</t>
+        </is>
+      </c>
+      <c r="B410" t="inlineStr">
+        <is>
+          <t>
++90 216 302 29 48</t>
+        </is>
+      </c>
+      <c r="C410" t="inlineStr">
+        <is>
+          <t>
+Sahrayı Cedit, Halk Sk. 5/A, 34734 Kadıköy/İstanbul, Türkiye</t>
+        </is>
+      </c>
+      <c r="D410" t="inlineStr">
+        <is>
+          <t>Kadikoy/Istanbul</t>
+        </is>
+      </c>
+      <c r="E410" t="inlineStr">
+        <is>
+          <t>2026-08-12 01:15</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
✅ Veri Güncellendi:  - Fri Aug 14 01:16:06 UTC 2026
</commit_message>
<xml_diff>
--- a/leads_output.xlsx
+++ b/leads_output.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E410"/>
+  <dimension ref="A1:E411"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -12308,6 +12308,35 @@
         </is>
       </c>
     </row>
+    <row r="411">
+      <c r="A411" t="inlineStr">
+        <is>
+          <t>Sarıyıldız Eczanesi</t>
+        </is>
+      </c>
+      <c r="B411" t="inlineStr">
+        <is>
+          <t>
++90 216 362 10 66</t>
+        </is>
+      </c>
+      <c r="C411" t="inlineStr">
+        <is>
+          <t>
+Bostancı, Prof. Dr. Kemal Akgüder Cd. No:1, 34744 Kadıköy/İstanbul, Türkiye</t>
+        </is>
+      </c>
+      <c r="D411" t="inlineStr">
+        <is>
+          <t>Kadikoy/Istanbul</t>
+        </is>
+      </c>
+      <c r="E411" t="inlineStr">
+        <is>
+          <t>2026-08-14 01:16</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
✅ Veri Güncellendi:  - Fri Aug 28 08:16:51 UTC 2026
</commit_message>
<xml_diff>
--- a/leads_output.xlsx
+++ b/leads_output.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E411"/>
+  <dimension ref="A1:E412"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -12337,6 +12337,35 @@
         </is>
       </c>
     </row>
+    <row r="412">
+      <c r="A412" t="inlineStr">
+        <is>
+          <t>Eczane Birol</t>
+        </is>
+      </c>
+      <c r="B412" t="inlineStr">
+        <is>
+          <t>
++90 216 338 58 95</t>
+        </is>
+      </c>
+      <c r="C412" t="inlineStr">
+        <is>
+          <t>
+Caferağa, Moda Cd. No:113, 34710 Kadıköy/İstanbul, Türkiye</t>
+        </is>
+      </c>
+      <c r="D412" t="inlineStr">
+        <is>
+          <t>Kadikoy/Istanbul</t>
+        </is>
+      </c>
+      <c r="E412" t="inlineStr">
+        <is>
+          <t>2026-08-28 08:16</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>